<commit_message>
vulcan and other changes
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 Villain Plan" sheetId="1" r:id="R8f67fb01529745e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rf7ee4ec6ea2c4d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rbf4a64d7e6014be8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="4" r:id="R27d6d10b340f4444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanic Templates" sheetId="5" r:id="R5586d26d1f274e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Summary" sheetId="6" r:id="Rbccb392b13314593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Audit" sheetId="7" r:id="R79bf5a2307c0450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 Villain Plan" sheetId="1" r:id="R276e927aa7834875"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rc9df6acf4aeb4b34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rc030a180b1394daa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="4" r:id="R93ebc1a983ee405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanic Templates" sheetId="5" r:id="R49f3316edebf4b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Summary" sheetId="6" r:id="Rda35a6e7f0444502"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Audit" sheetId="7" r:id="R5f342452d088479e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2171,217 +2171,145 @@
       </x:c>
     </x:row>
     <x:row r="15" s="25" customFormat="1" ht="68.0999984741211" customHeight="1">
-      <x:c r="A15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3 - Monsters</x:t>
-        </x:is>
+      <x:c r="A15" s="40" t="str">
+        <x:v>3 - Monsters</x:v>
       </x:c>
       <x:c r="B15" s="40" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Reptilla</x:t>
-        </x:is>
+      <x:c r="C15" s="40" t="str">
+        <x:v>Vulcan</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>Conner's Reptiles</x:v>
+        <x:v>Here Comes Trubble</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="F15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">In code - real/active mode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Playtest City Rampage pops, jackpot lighting, saucer 2 Super, timer reset, and case-file branches</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">reptilla</x:t>
-        </x:is>
+        <x:v>Corrected / verified</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>In code - real/active mode</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
+        <x:v>Playtest Vulcan heat/forge rules, gate/upper access, case-file branches, and chapter-fit as Monsters slot.</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>vulcan</x:v>
       </x:c>
       <x:c r="I15" s="40" t="str">
-        <x:v>https://marvelanimated.fandom.com/wiki/Reptilla_(Spider-Man_(1967))</x:v>
-      </x:c>
-      <x:c r="J15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Medium mode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pops rampage + jackpot shots</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pops build Rampage and jackpot value. Every 3 pops lights next Rampage Jackpot shot in order: left middle drop, upper middle target, right middle drop, then center web with More JPs.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pops, left middle drop setup, upper center target, right middle drop setup, center web, saucer 2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rampage jackpots score current value; Super at saucer 2 equals total collected rampage jackpots.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pop score rises 20K+1K to 50K; jackpot adds 25K/pop to 500K; Super timer is short and reset by pops.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adds 4th Rampage Jackpot at center web target.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rampage Jackpot awards 2X.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Super timer 10s -&gt; 16s.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10s ball save during Rampage.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shot Assist: first left-bank jackpot leaves all 3 left drops up and any left drop collects it.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="U15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chapter 3: rampage/pops and Super Pops bridge.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="V15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">High</x:t>
-        </x:is>
+        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
+        <x:v>Compact mode</x:v>
+      </x:c>
+      <x:c r="K15" s="40" t="str">
+        <x:v>Heat / forge</x:v>
+      </x:c>
+      <x:c r="L15" s="40" t="str">
+        <x:v>Build heat at spinner/pops, then forge jackpot at lit target before heat cools.</x:v>
+      </x:c>
+      <x:c r="M15" s="40" t="str">
+        <x:v>Spinner, pops, center target</x:v>
+      </x:c>
+      <x:c r="N15" s="40" t="str">
+        <x:v>Forge/cash heat jackpot.</x:v>
+      </x:c>
+      <x:c r="O15" s="40" t="str">
+        <x:v>Heat cools faster; more heat required.</x:v>
+      </x:c>
+      <x:c r="P15" s="40" t="str">
+        <x:v>+1 extra forge jackpot.</x:v>
+      </x:c>
+      <x:c r="Q15" s="40" t="str">
+        <x:v>+25% forged value.</x:v>
+      </x:c>
+      <x:c r="R15" s="40" t="str">
+        <x:v>+5s heat hold.</x:v>
+      </x:c>
+      <x:c r="S15" s="40" t="str">
+        <x:v>One overheat/drain protected.</x:v>
+      </x:c>
+      <x:c r="T15" s="40" t="str">
+        <x:v>Start with heat meter partly filled.</x:v>
+      </x:c>
+      <x:c r="U15" s="40" t="str">
+        <x:v>Chapter 3: fire/forge monster phase.</x:v>
+      </x:c>
+      <x:c r="V15" s="40" t="str">
+        <x:v>High</x:v>
       </x:c>
       <x:c r="W15" s="40" t="str">
-        <x:v>Reptilla is the intelligent reptile/alligator creature from Conner's Reptiles.</x:v>
+        <x:v>Moved into Monsters chapter; Vulcan appears in Here Comes Trubble as one of Miss Trubble's summoned figures.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="25" customFormat="1" ht="68.0999984741211" customHeight="1">
-      <x:c r="A16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3 - Monsters</x:t>
-        </x:is>
+      <x:c r="A16" s="40" t="str">
+        <x:v>3 - Monsters</x:v>
       </x:c>
       <x:c r="B16" s="40" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mole Man</x:t>
-        </x:is>
+      <x:c r="C16" s="40" t="str">
+        <x:v>Miss Trubble</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>Menace from the Bottom of the World / Spider-Man Battles the Molemen</x:v>
+        <x:v>Here Comes Trubble</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="F16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">In code - real/active mode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Playtest Find the Mole Man secret-target reveal, early-exit resets, hurry-up, and case-file branches</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">mole_man</x:t>
-        </x:is>
+        <x:v>Corrected / verified</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="str">
+        <x:v>In code - new/active mode</x:v>
+      </x:c>
+      <x:c r="G16" s="40" t="str">
+        <x:v>Playtest hidden-correct-shot reveal mode; tune reveal timing, wrong-shot limit, and shot pool</x:v>
+      </x:c>
+      <x:c r="H16" s="40" t="str">
+        <x:v>miss_trubble</x:v>
       </x:c>
       <x:c r="I16" s="40" t="str">
-        <x:v>https://en.wikipedia.org/wiki/List_of_Spider-Man_(1967_TV_series)_episodes</x:v>
-      </x:c>
-      <x:c r="J16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Medium mode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Upper reveal -&gt; secret drop target</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Enter upper; both banks reset; random secret lower drop target chosen. Upper targets drop non-secret targets while spinner builds value. Only secret remaining starts hurry-up.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Upper targets, upper spinner, both drop banks, bank rubbers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hit revealed secret target within hurry-up for jackpot.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Early upper exit or bad lower drop before reveal drops remaining targets and forces return upper; final hurry-up pressure.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">+1 extra/bonus hurry-up opportunity later if desired.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mole Man Jackpot 2X.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Secret-target hurry-up 16s -&gt; 24s.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10s ball save.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shot Assist: rubber on secret target's bank scores and drops the secret target programmatically.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="U16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chapter 3: hidden underground/search phase.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="V16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">High</x:t>
-        </x:is>
+        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
+      </x:c>
+      <x:c r="J16" s="40" t="str">
+        <x:v>Medium mode</x:v>
+      </x:c>
+      <x:c r="K16" s="40" t="str">
+        <x:v>Hidden correct shot / reveal</x:v>
+      </x:c>
+      <x:c r="L16" s="40" t="str">
+        <x:v>Each round selects 3 shot groups that look identical. One is correct and two are traps. Spinner briefly reveals correct shot bright green and bad shots dim red. Any selected shot ends the round and selects 3 new shots. Wrong shots add to a tally; 7 wrong shots ends mode.</x:v>
+      </x:c>
+      <x:c r="M16" s="40" t="str">
+        <x:v>Left web, center web, upper spinner, upper targets, drop banks, pops</x:v>
+      </x:c>
+      <x:c r="N16" s="40" t="str">
+        <x:v>Collect jackpots by choosing correct shots before 7 wrong choices.</x:v>
+      </x:c>
+      <x:c r="O16" s="40" t="str">
+        <x:v>Wrong-shot tally creates pressure; later rounds can use harder shot groups.</x:v>
+      </x:c>
+      <x:c r="P16" s="40" t="str">
+        <x:v>Adds 2 extra rounds.</x:v>
+      </x:c>
+      <x:c r="Q16" s="40" t="str">
+        <x:v>Increases jackpot value.</x:v>
+      </x:c>
+      <x:c r="R16" s="40" t="str">
+        <x:v>Spinner reveal lasts 2s instead of 750ms.</x:v>
+      </x:c>
+      <x:c r="S16" s="40" t="str">
+        <x:v>10s ball save at mode start.</x:v>
+      </x:c>
+      <x:c r="T16" s="40" t="str">
+        <x:v>First round: all 3 lit shots count as good/correct shots.</x:v>
+      </x:c>
+      <x:c r="U16" s="40" t="str">
+        <x:v>Chapter 3: Miss Trubble trick/trap reveal phase.</x:v>
+      </x:c>
+      <x:c r="V16" s="40" t="str">
+        <x:v>High</x:v>
       </x:c>
       <x:c r="W16" s="40" t="str">
-        <x:v>Molemen/Mole leader story family verified.</x:v>
+        <x:v>Moved into Monsters chapter; Miss Trubble is the main antagonist of Here Comes Trubble and anchors the Trubble Unleashed mini-wizard.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="25" customFormat="1" ht="68.0999984741211" customHeight="1">
@@ -2492,112 +2420,74 @@
       </x:c>
     </x:row>
     <x:row r="18" s="25" customFormat="1" ht="68.0999984741211" customHeight="1">
-      <x:c r="A18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4 - Crime Wave</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Miss Trubble</x:t>
-        </x:is>
+      <x:c r="A18" s="40" t="str">
+        <x:v>4 - Crime Wave</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>Mole Man</x:v>
       </x:c>
       <x:c r="D18" s="40" t="str">
-        <x:v>Here Comes Trubble</x:v>
+        <x:v>Menace from the Bottom of the World / Spider-Man Battles the Molemen</x:v>
       </x:c>
       <x:c r="E18" s="40" t="str">
-        <x:v>Corrected / verified</x:v>
-      </x:c>
-      <x:c r="F18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">In code - new/active mode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Playtest hidden-correct-shot reveal mode; tune reveal timing, wrong-shot limit, and shot pool</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">miss_trubble</x:t>
-        </x:is>
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="str">
+        <x:v>In code - real/active mode</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str">
+        <x:v>Playtest Find the Mole Man secret-target reveal, early-exit resets, hurry-up, and case-file branches</x:v>
+      </x:c>
+      <x:c r="H18" s="40" t="str">
+        <x:v>mole_man</x:v>
       </x:c>
       <x:c r="I18" s="40" t="str">
-        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
-      </x:c>
-      <x:c r="J18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Medium mode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hidden correct shot / reveal</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Each round selects 3 shot groups that look identical. One is correct and two are traps. Spinner briefly reveals correct shot bright green and bad shots dim red. Any selected shot ends the round and selects 3 new shots. Wrong shots add to a tally; 7 wrong shots ends mode.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Left web, center web, upper spinner, upper targets, drop banks, pops</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Collect jackpots by choosing correct shots before 7 wrong choices.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Wrong-shot tally creates pressure; later rounds can use harder shot groups.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adds 2 extra rounds.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Increases jackpot value.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Spinner reveal lasts 2s instead of 750ms.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10s ball save at mode start.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">First round: all 3 lit shots count as good/correct shots.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="U18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chapter 4: trick/trap-shot reveal phase.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="V18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">High</x:t>
-        </x:is>
+        <x:v>https://en.wikipedia.org/wiki/List_of_Spider-Man_(1967_TV_series)_episodes</x:v>
+      </x:c>
+      <x:c r="J18" s="40" t="str">
+        <x:v>Medium mode</x:v>
+      </x:c>
+      <x:c r="K18" s="40" t="str">
+        <x:v>Upper reveal -&gt; secret drop target</x:v>
+      </x:c>
+      <x:c r="L18" s="40" t="str">
+        <x:v>Enter upper; both banks reset; random secret lower drop target chosen. Upper targets drop non-secret targets while spinner builds value. Only secret remaining starts hurry-up.</x:v>
+      </x:c>
+      <x:c r="M18" s="40" t="str">
+        <x:v>Upper targets, upper spinner, both drop banks, bank rubbers</x:v>
+      </x:c>
+      <x:c r="N18" s="40" t="str">
+        <x:v>Hit revealed secret target within hurry-up for jackpot.</x:v>
+      </x:c>
+      <x:c r="O18" s="40" t="str">
+        <x:v>Early upper exit or bad lower drop before reveal drops remaining targets and forces return upper; final hurry-up pressure.</x:v>
+      </x:c>
+      <x:c r="P18" s="40" t="str">
+        <x:v>+1 extra/bonus hurry-up opportunity later if desired.</x:v>
+      </x:c>
+      <x:c r="Q18" s="40" t="str">
+        <x:v>Mole Man Jackpot 2X.</x:v>
+      </x:c>
+      <x:c r="R18" s="40" t="str">
+        <x:v>Secret-target hurry-up 16s -&gt; 24s.</x:v>
+      </x:c>
+      <x:c r="S18" s="40" t="str">
+        <x:v>10s ball save.</x:v>
+      </x:c>
+      <x:c r="T18" s="40" t="str">
+        <x:v>Shot Assist: rubber on secret target's bank scores and drops the secret target programmatically.</x:v>
+      </x:c>
+      <x:c r="U18" s="40" t="str">
+        <x:v>Chapter 4: hidden underground/search phase.</x:v>
+      </x:c>
+      <x:c r="V18" s="40" t="str">
+        <x:v>High</x:v>
       </x:c>
       <x:c r="W18" s="40" t="str">
-        <x:v>Miss Trubble is the main antagonist of Here Comes Trubble.</x:v>
+        <x:v>Moved from Monsters into Crime Wave; Molemen/Mole leader story family verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" s="25" customFormat="1" ht="68.0999984741211" customHeight="1">
@@ -3887,110 +3777,74 @@
       </x:c>
     </x:row>
     <x:row r="31" s="25" customFormat="1" ht="68.0999984741211" customHeight="1">
-      <x:c r="A31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6 - Mystic Menace</x:t>
-        </x:is>
+      <x:c r="A31" s="40" t="str">
+        <x:v>6 - Mystic Menace</x:v>
       </x:c>
       <x:c r="B31" s="40" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Vulcan</x:t>
-        </x:is>
+      <x:c r="C31" s="40" t="str">
+        <x:v>Reptilla</x:v>
       </x:c>
       <x:c r="D31" s="40" t="str">
-        <x:v>Here Comes Trubble</x:v>
+        <x:v>Conner's Reptiles</x:v>
       </x:c>
       <x:c r="E31" s="40" t="str">
-        <x:v>Corrected / verified</x:v>
-      </x:c>
-      <x:c r="F31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not in code</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Add placeholder only after confirming episode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">vulcan</x:t>
-        </x:is>
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="F31" s="40" t="str">
+        <x:v>In code - real/active mode</x:v>
+      </x:c>
+      <x:c r="G31" s="40" t="str">
+        <x:v>Playtest City Rampage pops, jackpot lighting, saucer 2 Super, timer reset, and case-file branches</x:v>
+      </x:c>
+      <x:c r="H31" s="40" t="str">
+        <x:v>reptilla</x:v>
       </x:c>
       <x:c r="I31" s="40" t="str">
-        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
-      </x:c>
-      <x:c r="J31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Compact mode</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Heat / forge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build heat at spinner/pops, then forge jackpot at lit target before heat cools.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Spinner, pops, center target</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Forge/cash heat jackpot.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Heat cools faster; more heat required.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">+1 extra forge jackpot.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">+25% forged value.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">+5s heat hold.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">One overheat/drain protected.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Start with heat meter partly filled.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="U31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chapter 6: fire/forge phase.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="V31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Low / verify</x:t>
-        </x:is>
+        <x:v>https://marvelanimated.fandom.com/wiki/Reptilla_(Spider-Man_(1967))</x:v>
+      </x:c>
+      <x:c r="J31" s="40" t="str">
+        <x:v>Medium mode</x:v>
+      </x:c>
+      <x:c r="K31" s="40" t="str">
+        <x:v>Pops rampage + jackpot shots</x:v>
+      </x:c>
+      <x:c r="L31" s="40" t="str">
+        <x:v>Pops build Rampage and jackpot value. Every 3 pops lights next Rampage Jackpot shot in order: left middle drop, upper middle target, right middle drop, then center web with More JPs.</x:v>
+      </x:c>
+      <x:c r="M31" s="40" t="str">
+        <x:v>Pops, left middle drop setup, upper center target, right middle drop setup, center web, saucer 2</x:v>
+      </x:c>
+      <x:c r="N31" s="40" t="str">
+        <x:v>Rampage jackpots score current value; Super at saucer 2 equals total collected rampage jackpots.</x:v>
+      </x:c>
+      <x:c r="O31" s="40" t="str">
+        <x:v>Pop score rises 20K+1K to 50K; jackpot adds 25K/pop to 500K; Super timer is short and reset by pops.</x:v>
+      </x:c>
+      <x:c r="P31" s="40" t="str">
+        <x:v>Adds 4th Rampage Jackpot at center web target.</x:v>
+      </x:c>
+      <x:c r="Q31" s="40" t="str">
+        <x:v>Rampage Jackpot awards 2X.</x:v>
+      </x:c>
+      <x:c r="R31" s="40" t="str">
+        <x:v>Super timer 10s -&gt; 16s.</x:v>
+      </x:c>
+      <x:c r="S31" s="40" t="str">
+        <x:v>10s ball save during Rampage.</x:v>
+      </x:c>
+      <x:c r="T31" s="40" t="str">
+        <x:v>Shot Assist: first left-bank jackpot leaves all 3 left drops up and any left drop collects it.</x:v>
+      </x:c>
+      <x:c r="U31" s="40" t="str">
+        <x:v>Chapter 6: creature/rampage phase.</x:v>
+      </x:c>
+      <x:c r="V31" s="40" t="str">
+        <x:v>High</x:v>
       </x:c>
       <x:c r="W31" s="40" t="str">
-        <x:v>Vulcan appears in Here Comes Trubble as one of Miss Trubble's summoned figures.</x:v>
+        <x:v>Moved out of Monsters into Mystic Menace; Reptilla is the intelligent reptile/alligator creature from Conner's Reptiles.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" s="25" customFormat="1" ht="68.0999984741211" customHeight="1">
@@ -7740,7 +7594,7 @@
         <x:v>Latest codebase</x:v>
       </x:c>
       <x:c r="B2" s="53" t="str">
-        <x:v>ASM67_2026_06_17c.zip</x:v>
+        <x:v>ASM67_2026_06_18a.zip + 18g chapter swap patch</x:v>
       </x:c>
       <x:c r="C2" s="40"/>
       <x:c r="D2" s="40"/>
@@ -7769,7 +7623,7 @@
         <x:v>Latest workbook update</x:v>
       </x:c>
       <x:c r="B3" s="53" t="str">
-        <x:v>2026-06-17 source verification pass</x:v>
+        <x:v>2026-06-18 chapter roster swap</x:v>
       </x:c>
       <x:c r="C3" s="40"/>
       <x:c r="D3" s="40"/>
@@ -7798,7 +7652,7 @@
         <x:v>Major corrections</x:v>
       </x:c>
       <x:c r="B4" s="53" t="str">
-        <x:v>Centaur/Cerberus/Cyclops/Vulcan -&gt; Here Comes Trubble; Reptilla -&gt; Conner's Reptiles; Doctor Manta -&gt; Phantom from the Depths of Time; Frederick Foswell -&gt; King Pinned; Sky Master -&gt; Criminals in the Clouds.</x:v>
+        <x:v>Monsters now uses Vulcan and Miss Trubble; Reptilla moved to Mystic Menace; Mole Man moved to Crime Wave; Chapter 3 mini-wizard renamed Trubble Unleashed.</x:v>
       </x:c>
       <x:c r="C4" s="40"/>
       <x:c r="D4" s="40"/>
@@ -7827,7 +7681,7 @@
         <x:v>Crime Wave status</x:v>
       </x:c>
       <x:c r="B5" s="53" t="str">
-        <x:v>Enforcers/Ox, Fifth Avenue Phantom, Frederick Foswell, Miss Trubble, Blackwell are designed/coded or in active test flow.</x:v>
+        <x:v>Enforcers/Ox, Mole Man, Fifth Avenue Phantom, Frederick Foswell, Blackwell are designed/coded or in active test flow.</x:v>
       </x:c>
       <x:c r="C5" s="40"/>
       <x:c r="D5" s="40"/>
@@ -7856,7 +7710,7 @@
         <x:v>Monsters status</x:v>
       </x:c>
       <x:c r="B6" s="53" t="str">
-        <x:v>Centaur, Cerberus, Cyclops, Reptilla, Mole Man are designed/coded or in active playtest flow.</x:v>
+        <x:v>Centaur, Cerberus, Cyclops, Vulcan, Miss Trubble are designed/coded or in active playtest flow.</x:v>
       </x:c>
       <x:c r="C6" s="40"/>
       <x:c r="D6" s="40"/>
@@ -7885,7 +7739,7 @@
         <x:v>Backups</x:v>
       </x:c>
       <x:c r="B7" s="53" t="str">
-        <x:v>Miss Trubble backup row marked duplicate/promoted; South Pole Natives and Pod verified as weak/theme/phase candidates.</x:v>
+        <x:v>Miss Trubble promoted to Monsters; Trubble Unleashed becomes the Monsters mini-wizard; Reptilla and Mole Man remain available in later chapters.</x:v>
       </x:c>
       <x:c r="C7" s="40"/>
       <x:c r="D7" s="40"/>
@@ -7943,7 +7797,7 @@
         <x:v>Mini-wizard flow</x:v>
       </x:c>
       <x:c r="B9" s="53" t="str">
-        <x:v>Placeholder mini-wizards use intro -&gt; VUK hold/release -&gt; 2-ball MB -&gt; summary -&gt; chapter advance.</x:v>
+        <x:v>Placeholder mini-wizards use intro -&gt; VUK hold/release -&gt; 2-ball MB -&gt; summary -&gt; chapter advance. Chapter 3 now opens gate for Trubble Unleashed when all 5 Monsters are complete.</x:v>
       </x:c>
       <x:c r="C9" s="40"/>
       <x:c r="D9" s="40"/>
@@ -7972,7 +7826,7 @@
         <x:v>Next work</x:v>
       </x:c>
       <x:c r="B10" s="53" t="str">
-        <x:v>Playtest latest ASM67 build, then finish remaining Chapter 4/5 designs or tune case-file/helper popups.</x:v>
+        <x:v>Playtest latest ASM67 build, then tune Chapter 3 Trubble Unleashed rules and finish remaining Chapter 4/5 designs.</x:v>
       </x:c>
       <x:c r="C10" s="40"/>
       <x:c r="D10" s="40"/>
@@ -12038,25 +11892,17 @@
           <x:t xml:space="preserve">3 - Monsters</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Monster Island Breakout</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The monsters escape together.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Centaur, Cerberus, Cyclops, Reptilla, Mole Man</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Placeholder 2-ball mini-wizard flow for now; later customize around monster attacks and area clears.</x:t>
-        </x:is>
+      <x:c r="B4" s="11" t="str">
+        <x:v>Trubble Unleashed</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>Miss Trubble unleashes her mythological monsters together.</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Centaur, Cerberus, Cyclops, Vulcan, Miss Trubble</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>Placeholder 2-ball mini-wizard flow for now; later customize around Miss Trubble commanding the monster attacks.</x:v>
       </x:c>
       <x:c r="F4" s="11" t="inlineStr">
         <x:is>
@@ -12109,10 +11955,8 @@
           <x:t xml:space="preserve">The Bugle exposes a citywide crime plan.</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Enforcers/Ox, Miss Trubble, Phantom, Foswell, Blackwell</x:t>
-        </x:is>
+      <x:c r="D5" s="11" t="str">
+        <x:v>Enforcers/Ox, Mole Man, Phantom, Foswell, Blackwell</x:v>
       </x:c>
       <x:c r="E5" s="11" t="inlineStr">
         <x:is>
@@ -12231,10 +12075,8 @@
           <x:t xml:space="preserve">Magic, mind control, and dimensions overlap.</x:t>
         </x:is>
       </x:c>
-      <x:c r="D7" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fakir rhythm, Kotep relics, Infinata loop, Pardo acts, Vulcan heat</x:t>
-        </x:is>
+      <x:c r="D7" s="11" t="str">
+        <x:v>Fakir rhythm, Kotep relics, Infinata loop, Pardo acts, Reptilla rampage</x:v>
       </x:c>
       <x:c r="E7" s="11" t="inlineStr">
         <x:is>
@@ -15721,16 +15563,16 @@
         <x:v>Latest codebase</x:v>
       </x:c>
       <x:c r="B2" s="53" t="str">
-        <x:v>ASM67_2026_06_17c.zip</x:v>
+        <x:v>ASM67_2026_06_18a.zip + 18g chapter swap patch</x:v>
       </x:c>
       <x:c r="C2" s="53" t="str">
-        <x:v>Workbook audit updated 2026-06-17</x:v>
+        <x:v>Workbook updated 2026-06-18 for chapter roster changes</x:v>
       </x:c>
       <x:c r="D2" s="53" t="str">
-        <x:v>Build future patches from this zip.</x:v>
+        <x:v>Build future patches from the current ASM67_2026_06_18a base plus applied changed-file patches.</x:v>
       </x:c>
       <x:c r="E2" s="53" t="str">
-        <x:v>Confirm local code matches workbook.</x:v>
+        <x:v>Confirm local code has the 18g chapter swap patch applied.</x:v>
       </x:c>
       <x:c r="F2" s="40" t="n"/>
       <x:c r="G2" s="40" t="n"/>
@@ -15756,16 +15598,16 @@
         <x:v>Monsters chapter</x:v>
       </x:c>
       <x:c r="B3" s="77" t="str">
-        <x:v>Centaur/Cerberus/Cyclops/Reptilla/Mole Man designed/coded</x:v>
+        <x:v>Centaur/Cerberus/Cyclops/Vulcan/Miss Trubble designed/coded</x:v>
       </x:c>
       <x:c r="C3" s="77" t="str">
-        <x:v>Centaur/Cyclops/Cerberus are Here Comes Trubble; Reptilla is Conner's Reptiles; Mole Man is Molemen episode family.</x:v>
+        <x:v>Centaur/Cyclops/Cerberus/Vulcan/Miss Trubble are tied to Here Comes Trubble; Miss Trubble anchors the chapter wizard.</x:v>
       </x:c>
       <x:c r="D3" s="77" t="str">
-        <x:v>Keep playtesting lights, bookends, widgets, case file helpers.</x:v>
+        <x:v>Keep playtesting lights, bookends, widgets, case-file helpers, gate/VUK wizard-ready flow.</x:v>
       </x:c>
       <x:c r="E3" s="77" t="str">
-        <x:v>Playtest all five.</x:v>
+        <x:v>Playtest all five and design custom Trubble Unleashed rules.</x:v>
       </x:c>
       <x:c r="F3" s="40" t="n"/>
       <x:c r="G3" s="40" t="n"/>
@@ -15791,10 +15633,10 @@
         <x:v>Crime Wave chapter</x:v>
       </x:c>
       <x:c r="B4" s="53" t="str">
-        <x:v>Enforcers/Ox, Miss Trubble, Fifth Avenue Phantom, Frederick Foswell, Blackwell current</x:v>
+        <x:v>Enforcers/Ox, Mole Man, Fifth Avenue Phantom, Frederick Foswell, Blackwell current</x:v>
       </x:c>
       <x:c r="C4" s="53" t="str">
-        <x:v>Foswell corrected to King Pinned; Enforcers/Ox to Blueprint for Crime; Phantom to Fifth Avenue Phantom/Dark Terrors.</x:v>
+        <x:v>Mole Man moved into Crime Wave; Foswell corrected to King Pinned; Enforcers/Ox to Blueprint for Crime; Phantom to Fifth Avenue Phantom/Dark Terrors.</x:v>
       </x:c>
       <x:c r="D4" s="58" t="str">
         <x:v>Cumulative Crime Wave work should be preserved in latest code.</x:v>
@@ -15861,10 +15703,10 @@
         <x:v>Oddities/backups</x:v>
       </x:c>
       <x:c r="B6" s="53" t="str">
-        <x:v>Some rows are better as phases/themes</x:v>
+        <x:v>Some rows are better as phases/themes; Miss Trubble backup remains duplicate/promoted</x:v>
       </x:c>
       <x:c r="C6" s="53" t="str">
-        <x:v>Pod = Rollarama hazard; South Pole Natives = Neptune's Nose Cone setting; Miss Trubble backup duplicate.</x:v>
+        <x:v>Pod = Rollarama hazard; South Pole Natives = Neptune's Nose Cone setting; Miss Trubble backup duplicate/promoted to Monsters.</x:v>
       </x:c>
       <x:c r="D6" s="58" t="str">
         <x:v>Do not promote weak/theme rows until needed.</x:v>
@@ -18352,25 +18194,25 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>Reptilla</x:v>
+        <x:v>Vulcan</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>Conner's Reptiles</x:v>
+        <x:v>Here Comes Trubble</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Corrected / verified</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>https://marvelanimated.fandom.com/wiki/Reptilla_(Spider-Man_(1967))</x:v>
+        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
-        <x:v>Reptilla is the intelligent reptile/alligator creature from Conner's Reptiles.</x:v>
+        <x:v>Moved into Monsters; Vulcan appears in Here Comes Trubble as one of Miss Trubble's summoned figures.</x:v>
       </x:c>
       <x:c r="G15" s="40" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H15" s="40" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Moved</x:v>
       </x:c>
       <x:c r="I15" s="40"/>
       <x:c r="J15" s="40"/>
@@ -18393,25 +18235,25 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="40" t="str">
-        <x:v>Mole Man</x:v>
+        <x:v>Miss Trubble</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>Menace from the Bottom of the World / Spider-Man Battles the Molemen</x:v>
+        <x:v>Here Comes Trubble</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Corrected / verified</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>https://en.wikipedia.org/wiki/List_of_Spider-Man_(1967_TV_series)_episodes</x:v>
+        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>Molemen/Mole leader story family verified.</x:v>
+        <x:v>Moved into Monsters; Miss Trubble anchors the Trubble Unleashed mini-wizard.</x:v>
       </x:c>
       <x:c r="G16" s="40" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H16" s="40" t="str">
-        <x:v>Verified</x:v>
+        <x:v>Moved</x:v>
       </x:c>
       <x:c r="I16" s="40"/>
       <x:c r="J16" s="40"/>
@@ -18475,25 +18317,25 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="40" t="str">
-        <x:v>Miss Trubble</x:v>
+        <x:v>Mole Man</x:v>
       </x:c>
       <x:c r="C18" s="40" t="str">
-        <x:v>Here Comes Trubble</x:v>
+        <x:v>Menace from the Bottom of the World / Spider-Man Battles the Molemen</x:v>
       </x:c>
       <x:c r="D18" s="40" t="str">
-        <x:v>Corrected / verified</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="E18" s="40" t="str">
-        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
+        <x:v>https://en.wikipedia.org/wiki/List_of_Spider-Man_(1967_TV_series)_episodes</x:v>
       </x:c>
       <x:c r="F18" s="40" t="str">
-        <x:v>Miss Trubble is the main antagonist of Here Comes Trubble.</x:v>
+        <x:v>Moved into Crime Wave; Molemen/Mole leader story family verified.</x:v>
       </x:c>
       <x:c r="G18" s="40" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H18" s="40" t="str">
-        <x:v>Corrected</x:v>
+        <x:v>Moved</x:v>
       </x:c>
       <x:c r="I18" s="40"/>
       <x:c r="J18" s="40"/>
@@ -19008,25 +18850,25 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B31" s="40" t="str">
-        <x:v>Vulcan</x:v>
+        <x:v>Reptilla</x:v>
       </x:c>
       <x:c r="C31" s="40" t="str">
-        <x:v>Here Comes Trubble</x:v>
+        <x:v>Conner's Reptiles</x:v>
       </x:c>
       <x:c r="D31" s="40" t="str">
-        <x:v>Corrected / verified</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="E31" s="40" t="str">
-        <x:v>https://marvel.fandom.com/wiki/Spider-Man_(1967_animated_series)_Season_1_11B</x:v>
+        <x:v>https://marvelanimated.fandom.com/wiki/Reptilla_(Spider-Man_(1967))</x:v>
       </x:c>
       <x:c r="F31" s="40" t="str">
-        <x:v>Vulcan appears in Here Comes Trubble as one of Miss Trubble's summoned figures.</x:v>
+        <x:v>Moved into Mystic Menace; Reptilla is the intelligent reptile/alligator creature from Conner's Reptiles.</x:v>
       </x:c>
       <x:c r="G31" s="40" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="H31" s="40" t="str">
-        <x:v>Corrected</x:v>
+        <x:v>Moved</x:v>
       </x:c>
       <x:c r="I31" s="40"/>
       <x:c r="J31" s="40"/>

</xml_diff>

<commit_message>
message tweaks for 1st 10
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R620ead94cdbc4de8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R01d47932221b49ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rb8b9b74541014010"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R79432deca8e44e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R5ffc64d6d5a5487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R0f23334e01be442d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R436c49dfab8e45f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Ra025beeb449d4e48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rabb03f7ed7e04acf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R4e83b5fd9186414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3d0358e813db4d56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R30b0596b39c6490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R4d85dc587d3748c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R10ab0a437ec64204"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rd2e174fa22e84714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R3a0fb56df5134868"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rfee91541f7274e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R0d03cd605e6d49b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R8b813465bd794752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R0b6965da85da45a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4996,16 +4996,16 @@
         <x:v>2-ball MB</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Chaos multiball: chase solid/flashing windows and saucer/shot opportunities.</x:v>
+        <x:v>Chaos multiball alternates between uncontrolled chaos and a calm saucer-held attack window.</x:v>
       </x:c>
       <x:c r="G7" t="str">
         <x:v>Ends when multiball ends, or when Goblin objectives complete if reached first.</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>Chaos multiball; windows alternate between solid/flashing scoring; banks goblin_bonus.</x:v>
+        <x:v>During chaos, STAR, pops, web targets, and drops reduce the Chaos Bonus. A saucer hold calms the mode and lights those shots for Goblin Jackpots. Jackpot starts at 100K, rises 50K per collect to 500K, and each collect also banks the same amount into Chaos Bonus.</x:v>
       </x:c>
       <x:c r="I7" s="31" t="str">
-        <x:v>Improved: persistent flashing/solid shot counts and stabilized bank status.</x:v>
+        <x:v>Redesigned: persistent Chaos Bonus, saucer-controlled calm windows, growing Goblin Jackpot, and no spinner scoring.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5034,7 +5034,7 @@
         <x:v>Rollovers lock arms; completing left bank locks one arm and enables jackpots; spinner boosts multiplier.</x:v>
       </x:c>
       <x:c r="I8" s="31" t="str">
-        <x:v>Improved: persistent arm-lock, web-jackpot, and breakout progress.</x:v>
+        <x:v>Adjusted: spinner flashes when active, arm-release timer resets on new locks, obsolete jackpot widget removed.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5063,7 +5063,7 @@
         <x:v>Hidden Super/clue mode; wrong shots score smaller and reduce value; clues narrow the target.</x:v>
       </x:c>
       <x:c r="I9" s="31" t="str">
-        <x:v>Improved: persistent remaining-shot count and current Super value.</x:v>
+        <x:v>Adjusted: non-clue shots now post a generic Mysterio callout event; recording still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5092,7 +5092,7 @@
         <x:v>Spinner builds Venom; upper exit stages timed drop-bank attack shots.</x:v>
       </x:c>
       <x:c r="I10" s="31" t="str">
-        <x:v>Improved: persistent Venom build, attempt count, exit choice, and staged target status.</x:v>
+        <x:v>Adjusted: exact roof-spinner objective, reusable reminder flag, and delayed Jackpot-to-next-objective pacing.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -5121,7 +5121,7 @@
         <x:v>Heat-area multiball; left/right/pops build heat; maxed areas light saucer jackpots and add-a-ball opportunities.</x:v>
       </x:c>
       <x:c r="I11" s="31" t="str">
-        <x:v>Improved: persistent lit-saucer and collected-jackpot totals.</x:v>
+        <x:v>Adjusted: meaningful saucer/jackpot status, ordinary zone-hit scoring, and delayed BALL ADDED message.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">

</xml_diff>

<commit_message>
swami, kotep (scarlet), and infinata (frog ghosts)
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R301a2d3c4aa24c18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rb4a9c5d0469040d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R1704807c2d294fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R921c5c2296264c81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R23c16ff87bf84640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R1775bfe0b3094214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R5962fc067a6d4d17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R1e46bd8294614cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R91331fac76314a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Ra229a1d4d12b4b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R29f07465886e411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R64c33406e0884199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Re9dcdc7410474c84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rcfdd75f3c2b04018"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R94bb59b431504d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Red4f86dabe0e440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R5ee4fc0fe8e74535"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R2830971c099c4da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Ra2924fee33b147f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rf4c99f4ce9154104"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1571,31 +1571,31 @@
         <x:v>Super Swami</x:v>
       </x:c>
       <x:c r="E25" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F25" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>Build-and-cash</x:v>
+        <x:v>Timed / urgency</x:v>
       </x:c>
       <x:c r="H25" t="str">
-        <x:v>Bonus-bank candidate</x:v>
+        <x:v>Area restoration</x:v>
       </x:c>
       <x:c r="I25" t="str">
-        <x:v>Landmark/objective shots</x:v>
+        <x:v>Six coordinate-based playfield regions</x:v>
       </x:c>
       <x:c r="J25" t="str">
-        <x:v>super_swami_bonus bank</x:v>
+        <x:v>Increasing restoration jackpots</x:v>
       </x:c>
       <x:c r="K25" t="str">
-        <x:v>Objective routing / disappearing values</x:v>
+        <x:v>40-second city blackout; 50 seconds with More Time</x:v>
       </x:c>
       <x:c r="L25" t="str">
-        <x:v>Goals completed / ball end</x:v>
+        <x:v>All 6 areas restored / timer expired / ball end</x:v>
       </x:c>
       <x:c r="M25" t="str">
-        <x:v>Chapter 5 banked-bonus role; should feel different from Fakir MB.</x:v>
+        <x:v>Simple Mystic Menace timed mode. Shot Assist spots one extra area; Safety Net starts ball save; More Jackpots adds a 500K VUK Blackout Jackpot.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1606,37 +1606,37 @@
         <x:v>Mystic Menace</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>frog_ghosts</x:v>
+        <x:v>infinata</x:v>
       </x:c>
       <x:c r="D26" t="str">
-        <x:v>Frog Ghosts</x:v>
+        <x:v>Infinata</x:v>
       </x:c>
       <x:c r="E26" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F26" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>Movement / chaos</x:v>
+        <x:v>Sequential area completion</x:v>
       </x:c>
       <x:c r="H26" t="str">
-        <x:v>Jumping target candidate</x:v>
+        <x:v>Pops, left drops, right drops, webs, upper targets</x:v>
       </x:c>
       <x:c r="I26" t="str">
-        <x:v>Pops + target groups</x:v>
+        <x:v>Rising area awards and timed saucer Super</x:v>
       </x:c>
       <x:c r="J26" t="str">
-        <x:v>Jumping jackpots / combo values</x:v>
+        <x:v>One green area at a time; 20-second Super timer</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>Moving target pressure</x:v>
+        <x:v>Saucer Super collected / timer expired / ball end</x:v>
       </x:c>
       <x:c r="L26" t="str">
-        <x:v>Goals or timer / ball end</x:v>
+        <x:v>Three areas required; optional fourth with More Jackpots</x:v>
       </x:c>
       <x:c r="M26" t="str">
-        <x:v>Should be the strange/chaotic movement mode in Mystic Menace.</x:v>
+        <x:v>Case files: 4th area, larger values, 30s Super timer, ball save, first hit awards two areas.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -3473,10 +3473,10 @@
         <x:v>Super Swami</x:v>
       </x:c>
       <x:c r="G25" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="H25" s="31" t="str">
-        <x:v>Chapter 5 bonus-bank candidate; uses super_swami_bonus naming.</x:v>
+        <x:v>40-second Restore New York mode. GI starts at 404040. Any valid switch in each of six monitor-coordinate regions restores that area permanently. Area awards start at 100K and rise 50K each; More Time gives 50 seconds and Bigger Jackpots starts at 200K.</x:v>
       </x:c>
       <x:c r="I25" s="31" t="str">
         <x:v>fifth_dimension_curse</x:v>
@@ -3499,16 +3499,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="E26" s="31" t="str">
-        <x:v>frog_ghosts</x:v>
+        <x:v>infinata</x:v>
       </x:c>
       <x:c r="F26" s="31" t="str">
-        <x:v>Frog Ghosts</x:v>
+        <x:v>Infinata</x:v>
       </x:c>
       <x:c r="G26" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="H26" s="31" t="str">
-        <x:v>Needs full Mystic Menace design.</x:v>
+        <x:v>One green creature area lights at a time. Complete three areas, then collect a timed Super Jackpot at any saucer. More Jackpots adds a fourth optional green area during the Super countdown.</x:v>
       </x:c>
       <x:c r="I26" s="31" t="str">
         <x:v>fifth_dimension_curse</x:v>
@@ -5617,6 +5617,64 @@
         <x:v>Improved: persistent left/right drop progress and live spinner value.</x:v>
       </x:c>
     </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="31" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B30" s="31" t="str">
+        <x:v>Mystic Menace</x:v>
+      </x:c>
+      <x:c r="C30" s="31" t="str">
+        <x:v>super_swami</x:v>
+      </x:c>
+      <x:c r="D30" s="31" t="str">
+        <x:v>Super Swami</x:v>
+      </x:c>
+      <x:c r="E30" s="31" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F30" s="31" t="str">
+        <x:v>GI dims to 404040; hit any valid switch in each of six physical playfield regions to restore New York.</x:v>
+      </x:c>
+      <x:c r="G30" s="31" t="str">
+        <x:v>Ends when all six areas are restored, the timer expires, or the ball ends. With More Jackpots, a final 500K VUK collect is required.</x:v>
+      </x:c>
+      <x:c r="H30" s="31" t="str">
+        <x:v>Base timer 40s, or 50s with More Time. Area values are 100K–350K, or 200K–450K with Bigger Jackpots. Restored areas stay lit.</x:v>
+      </x:c>
+      <x:c r="I30" s="31" t="str">
+        <x:v>Implemented: live area progress, countdown, restoration messages, case-file helpers, drop resets, and saucer kickouts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="31" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B31" s="31" t="str">
+        <x:v>Mystic Menace</x:v>
+      </x:c>
+      <x:c r="C31" s="31" t="str">
+        <x:v>infinata</x:v>
+      </x:c>
+      <x:c r="D31" s="31" t="str">
+        <x:v>Infinata</x:v>
+      </x:c>
+      <x:c r="E31" s="31" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F31" s="31" t="str">
+        <x:v>Clear one green creature area at a time. Areas are selected from pops, left drops, right drops, webs, and upper targets.</x:v>
+      </x:c>
+      <x:c r="G31" s="31" t="str">
+        <x:v>After three area completions, all three saucers light for a timed Super. Ends on Super collect, timer expiry, or ball end.</x:v>
+      </x:c>
+      <x:c r="H31" s="31" t="str">
+        <x:v>Area awards are 200K, 300K, 400K; Super is 1M. Bigger Jackpots raises values. More Time extends the Super from 20s to 30s.</x:v>
+      </x:c>
+      <x:c r="I31" s="31" t="str">
+        <x:v>More Jackpots adds a fourth optional green area during the Super countdown. Shot Assist makes the first valid hit award the active and next areas.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
5th dim wiz, case file add to jps
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R29f07465886e411d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R64c33406e0884199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Re9dcdc7410474c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rcfdd75f3c2b04018"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R94bb59b431504d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Red4f86dabe0e440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R5ee4fc0fe8e74535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R2830971c099c4da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Ra2924fee33b147f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rf4c99f4ce9154104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra6689fc2c1e54587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rb4ff5d2bcb8943f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R416818b8ef554d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R4f8eaa3ee7c443e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R1aa7dc55db8146cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Ra069c3f268174b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R35a5f93c6d08484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Ra7738754269040c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R7a328d1046504cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R2d4e645c7d364c5a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4383,7 +4383,7 @@
         <x:v>start_mode_sinister_surge</x:v>
       </x:c>
       <x:c r="F2" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G2" s="31" t="str">
         <x:v>Implemented; needs continued playtest/polish.</x:v>
@@ -4406,7 +4406,7 @@
         <x:v>start_mode_mastermind_trap</x:v>
       </x:c>
       <x:c r="F3" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G3" s="31" t="str">
         <x:v>Implemented; trap objectives and multiball scoring present.</x:v>
@@ -4429,7 +4429,7 @@
         <x:v>start_mode_trubble_unleashed</x:v>
       </x:c>
       <x:c r="F4" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G4" s="31" t="str">
         <x:v>Implemented; staged drops, saucers, VUK add-a-ball and multiball flow present.</x:v>
@@ -4452,7 +4452,7 @@
         <x:v>start_mode_master_plan</x:v>
       </x:c>
       <x:c r="F5" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G5" s="31" t="str">
         <x:v>Implemented; headlines/schemes/Daily Bugle super flow present.</x:v>
@@ -4475,10 +4475,10 @@
         <x:v>start_mode_fifth_dimension_curse</x:v>
       </x:c>
       <x:c r="F6" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G6" s="31" t="str">
-        <x:v>Placeholder/simple wizard; needs full design.</x:v>
+        <x:v>Implemented / needs playtest. Starts 3-ball multiball. Six GI zones stay bright 5s, flicker 3s, then dim independently. VUK jackpots score 500K–1.75M from active zones without clearing them. Upper targets score 100K + 25K per active zone, cycle purple pulse/solid/three flashes, and can award up to three add-a-balls after 3+ zone jackpots. Ends when down to one ball.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4498,7 +4498,7 @@
         <x:v>start_mode_mad_science_meltdown</x:v>
       </x:c>
       <x:c r="F7" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G7" s="31" t="str">
         <x:v>Placeholder/simple wizard; needs full design.</x:v>
@@ -4521,7 +4521,7 @@
         <x:v>start_mode_nature_strikes_back</x:v>
       </x:c>
       <x:c r="F8" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G8" s="31" t="str">
         <x:v>Placeholder/simple wizard; needs full design.</x:v>
@@ -4544,7 +4544,7 @@
         <x:v>start_mode_invasion_from_everywhere</x:v>
       </x:c>
       <x:c r="F9" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G9" s="31" t="str">
         <x:v>Placeholder/simple wizard; needs full design.</x:v>
@@ -4567,7 +4567,7 @@
         <x:v>start_mode_who_is_the_real_villain</x:v>
       </x:c>
       <x:c r="F10" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G10" s="31" t="str">
         <x:v>Placeholder/simple wizard; needs full design.</x:v>
@@ -4590,7 +4590,7 @@
         <x:v>start_mode_time_tossed_showdown</x:v>
       </x:c>
       <x:c r="F11" s="31" t="str">
-        <x:v>Uses chapter case-file total 0–25 for values; active case-file powers are not used.</x:v>
+        <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, target, spinner, progress, trap-completion, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G11" s="31" t="str">
         <x:v>Placeholder/simple wizard; needs full design.</x:v>

</xml_diff>

<commit_message>
music changes, more modes
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0689e904d5ff48ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rccb6b37421474cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R72f780dea59e4f4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R78077cae36ec4db9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R524312a8e4ed402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Re6064498c2174a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rc1d72e82af614645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Re13f02e8309f4adf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Ree8dd6649a844779"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rc64532a5eeaf4f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rb0d01bc622d64135"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R488963cebe844f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8681d20a12c54d9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R1f64d79bd9344cbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rdd10dcc57a9e44fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R77881bc7750e40be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rb017133334ef40e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Raafefa16eefb4d4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R62ea8e3523a5400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R9891d68e1da54bcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rd8727351b67448d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R1b900bb4a95242c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rd21a5303022146d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R7c0f7bc9041e4ac9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R29a08e63619a4995"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +25,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="9">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -75,8 +76,19 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -118,15 +130,51 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="5">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="81">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -263,6 +311,57 @@
     <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -371,9 +470,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2146,37 +2245,37 @@
         <x:v>Elemental Chaos</x:v>
       </x:c>
       <x:c r="C38" s="31" t="str">
-        <x:v>dr_zap</x:v>
+        <x:v>dr_zapp</x:v>
       </x:c>
       <x:c r="D38" s="31" t="str">
         <x:v>Doctor Zapp</x:v>
       </x:c>
       <x:c r="E38" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F38" s="31" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G38" s="31" t="str">
-        <x:v>Electrical machine / timed</x:v>
+        <x:v>Qualification / spinner attack</x:v>
       </x:c>
       <x:c r="H38" s="31" t="str">
-        <x:v>Invention control</x:v>
+        <x:v>Upper-target multiplier</x:v>
       </x:c>
       <x:c r="I38" s="31" t="str">
-        <x:v>Spinner + lit shots</x:v>
+        <x:v>Lower banks + rooftop spinner/targets</x:v>
       </x:c>
       <x:c r="J38" s="31" t="str">
-        <x:v>Zapp/Super value</x:v>
+        <x:v>100K drops; 50K helpers/flashes</x:v>
       </x:c>
       <x:c r="K38" s="31" t="str">
-        <x:v>Overload timing</x:v>
+        <x:v>Must qualify roof access and build flashes under active play</x:v>
       </x:c>
       <x:c r="L38" s="31" t="str">
-        <x:v>Sequence complete / timer / ball end</x:v>
+        <x:v>25 flashes / ball end</x:v>
       </x:c>
       <x:c r="M38" s="31" t="str">
-        <x:v>Must stay distinct from Electro by focusing on Caldwell's stolen invention.</x:v>
+        <x:v>Distinct from Electro: fixed rooftop camera-flash objective with helper targets rather than a travelling playfield spark.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2187,37 +2286,37 @@
         <x:v>Elemental Chaos</x:v>
       </x:c>
       <x:c r="C39" s="31" t="str">
-        <x:v>voltan_boomer</x:v>
+        <x:v>bolton_boomer</x:v>
       </x:c>
       <x:c r="D39" s="31" t="str">
-        <x:v>Voltan and Boomer</x:v>
+        <x:v>Bolton and Boomer</x:v>
       </x:c>
       <x:c r="E39" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F39" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G39" s="31" t="str">
-        <x:v>Storm timing / robbery</x:v>
+        <x:v>Capture-loop multiball</x:v>
       </x:c>
       <x:c r="H39" s="31" t="str">
-        <x:v>Thunder windows</x:v>
+        <x:v>Timed Super Jackpot</x:v>
       </x:c>
       <x:c r="I39" s="31" t="str">
-        <x:v>Storm shots + target groups</x:v>
+        <x:v>Random target + saucers + VUK</x:v>
       </x:c>
       <x:c r="J39" s="31" t="str">
-        <x:v>Thunder/robbery jackpots</x:v>
+        <x:v>Capture-loop jackpots and escalating Supers</x:v>
       </x:c>
       <x:c r="K39" s="31" t="str">
-        <x:v>Short storm windows</x:v>
+        <x:v>One ball is captured while the other must reach the VUK; later Supers are timed</x:v>
       </x:c>
       <x:c r="L39" s="31" t="str">
-        <x:v>Goals completed / ball end</x:v>
+        <x:v>Super sequence complete / multiball end</x:v>
       </x:c>
       <x:c r="M39" s="31" t="str">
-        <x:v>Thunder Rumble pair kept together; full design pending.</x:v>
+        <x:v>Repeating target-capture-release loop; unlike Dr. Manta, both balls participate in a conventional ongoing multiball.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2316,31 +2415,31 @@
         <x:v>Dr. Manta</x:v>
       </x:c>
       <x:c r="E42" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F42" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>2 staged / 1 active</x:v>
       </x:c>
       <x:c r="G42" s="31" t="str">
-        <x:v>Hidden-city control</x:v>
+        <x:v>Relay / staged ball control</x:v>
       </x:c>
       <x:c r="H42" s="31" t="str">
-        <x:v>Trap / freeze</x:v>
+        <x:v>Timed jackpot build-and-cash</x:v>
       </x:c>
       <x:c r="I42" s="31" t="str">
-        <x:v>Saucers + robotic-creature shots</x:v>
+        <x:v>VUK, three saucers, both spinners, upper targets</x:v>
       </x:c>
       <x:c r="J42" s="31" t="str">
-        <x:v>Frozen-city jackpots</x:v>
+        <x:v>100K VUK; 150K saucer; 100K starting JP; +50K/spin to 1M; repeated upper-target collections</x:v>
       </x:c>
       <x:c r="K42" s="31" t="str">
-        <x:v>Held ball / trap pressure</x:v>
+        <x:v>Second ball must reach a saucer; active attack ball may leave the roof; all flippers disable at timeout</x:v>
       </x:c>
       <x:c r="L42" s="31" t="str">
-        <x:v>Goals or timer / ball end</x:v>
+        <x:v>Attack timer expires and active ball reaches trough / early second-ball loss</x:v>
       </x:c>
       <x:c r="M42" s="31" t="str">
-        <x:v>Main Phantom from the Depths of Time villain.</x:v>
+        <x:v>Mechanically distinct from Molemen: never conventional free two-ball play after setup. One ball is always held while the other performs the objective.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2477,34 +2576,34 @@
         <x:v>molemen</x:v>
       </x:c>
       <x:c r="D46" s="31" t="str">
-        <x:v>Molemen</x:v>
+        <x:v>The Molemen</x:v>
       </x:c>
       <x:c r="E46" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F46" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G46" s="31" t="str">
-        <x:v>Underground invasion</x:v>
+        <x:v>Area-control multiball</x:v>
       </x:c>
       <x:c r="H46" s="31" t="str">
-        <x:v>Area / survival</x:v>
+        <x:v>Saucer jackpots / add-a-ball</x:v>
       </x:c>
       <x:c r="I46" s="31" t="str">
-        <x:v>Drops, tunnels, lower playfield</x:v>
+        <x:v>Left pop, center web, right pop + three saucers</x:v>
       </x:c>
       <x:c r="J46" s="31" t="str">
-        <x:v>Underground jackpots</x:v>
+        <x:v>50K pops; 100K center; 250K per ball saucer jackpots</x:v>
       </x:c>
       <x:c r="K46" s="31" t="str">
-        <x:v>Escalating underground pressure</x:v>
+        <x:v>Jackpot value depends on balls in play; each area offers one add-a-ball; short one-ball grace</x:v>
       </x:c>
       <x:c r="L46" s="31" t="str">
-        <x:v>Goals or timer / ball end</x:v>
+        <x:v>One-ball grace expires / ball end</x:v>
       </x:c>
       <x:c r="M46" s="31" t="str">
-        <x:v>Compact mode name; Mugs Reilly can appear in intro and summaries.</x:v>
+        <x:v>Chapter 9's conventional area-control multiball. It contrasts with Dr. Manta's staged relay, where one ball is always deliberately held.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -3522,10 +3621,10 @@
         <x:v>Elemental Chaos</x:v>
       </x:c>
       <x:c r="B9" s="31" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="31" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="31" t="str">
         <x:v>Nature Strikes Back</x:v>
@@ -3560,10 +3659,10 @@
         <x:v>Lost Worlds</x:v>
       </x:c>
       <x:c r="B10" s="31" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C10" s="31" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="31" t="str">
         <x:v>Invasion from Everywhere</x:v>
@@ -3649,6 +3748,1217 @@
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="63" t="str">
+        <x:v>ASM67 Music Inventory — Rebalanced Coded Assignments</x:v>
+      </x:c>
+      <x:c r="B1" s="63"/>
+      <x:c r="C1" s="63"/>
+      <x:c r="D1" s="63"/>
+      <x:c r="E1" s="63"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="67" t="str">
+        <x:v>Source of truth: ASM67_2026_08_06_1am plus this music patch. villain_bookends.py is canonical for villain/wizard gameplay music.</x:v>
+      </x:c>
+      <x:c r="B2" s="67"/>
+      <x:c r="C2" s="67"/>
+      <x:c r="D2" s="67"/>
+      <x:c r="E2" s="67"/>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="67" t="str">
+        <x:v>Rule: every villain/wizard gameplay song has at most two uses. maintheme, loop*, and intro_* tracks do not soundtrack villain/wizard gameplay; shared transition/core uses may remain.</x:v>
+      </x:c>
+      <x:c r="B3" s="67"/>
+      <x:c r="C3" s="67"/>
+      <x:c r="D3" s="67"/>
+      <x:c r="E3" s="67"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="72" t="str">
+        <x:v>Song #</x:v>
+      </x:c>
+      <x:c r="B5" s="72" t="str">
+        <x:v>Configured Asset</x:v>
+      </x:c>
+      <x:c r="C5" s="72" t="str">
+        <x:v>Effective Uses</x:v>
+      </x:c>
+      <x:c r="D5" s="72" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+      <x:c r="E5" s="72" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="74" t="str">
+        <x:v>prowl_car</x:v>
+      </x:c>
+      <x:c r="C6" s="74" t="str">
+        <x:v>Main play random pool</x:v>
+      </x:c>
+      <x:c r="D6" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="74" t="str"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="74" t="str">
+        <x:v>panic_patrol</x:v>
+      </x:c>
+      <x:c r="C7" s="74" t="str">
+        <x:v>Main play random pool</x:v>
+      </x:c>
+      <x:c r="D7" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="74" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="73" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="74" t="str">
+        <x:v>rat_race</x:v>
+      </x:c>
+      <x:c r="C8" s="74" t="str">
+        <x:v>Cyclops; Kingpin / Final Showdown</x:v>
+      </x:c>
+      <x:c r="D8" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E8" s="74" t="str"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="73" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="74" t="str">
+        <x:v>ticking</x:v>
+      </x:c>
+      <x:c r="C9" s="74" t="str">
+        <x:v>Green Lizard</x:v>
+      </x:c>
+      <x:c r="D9" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="74" t="str"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="73" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="74" t="str">
+        <x:v>start_loop</x:v>
+      </x:c>
+      <x:c r="C10" s="74" t="str">
+        <x:v>Ball start / skill-shot lead-in</x:v>
+      </x:c>
+      <x:c r="D10" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="74" t="str"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="73" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="74" t="str">
+        <x:v>maintheme_no_lyrics</x:v>
+      </x:c>
+      <x:c r="C11" s="74" t="str">
+        <x:v>Bonus; High Score</x:v>
+      </x:c>
+      <x:c r="D11" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E11" s="74" t="str">
+        <x:v>Protected main-theme variant; no villain/wizard gameplay use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="73" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B12" s="74" t="str">
+        <x:v>dash_to_safety</x:v>
+      </x:c>
+      <x:c r="C12" s="74" t="str">
+        <x:v>Green Goblin</x:v>
+      </x:c>
+      <x:c r="D12" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="74" t="str"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="73" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B13" s="74" t="str">
+        <x:v>cloak</x:v>
+      </x:c>
+      <x:c r="C13" s="74" t="str">
+        <x:v>Sandman; Dr. Von Schlick</x:v>
+      </x:c>
+      <x:c r="D13" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E13" s="74" t="str"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="73" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B14" s="74" t="str">
+        <x:v>fright</x:v>
+      </x:c>
+      <x:c r="C14" s="74" t="str">
+        <x:v>Skymaster; main play random pool</x:v>
+      </x:c>
+      <x:c r="D14" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E14" s="74" t="str"/>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="73" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B15" s="74" t="str">
+        <x:v>fromthebird</x:v>
+      </x:c>
+      <x:c r="C15" s="74" t="str">
+        <x:v>Vulture</x:v>
+      </x:c>
+      <x:c r="D15" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E15" s="74" t="str"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="77" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B16" s="78" t="str">
+        <x:v>intro_loop_2</x:v>
+      </x:c>
+      <x:c r="C16" s="78" t="str"/>
+      <x:c r="D16" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="78" t="str">
+        <x:v>Protected intro_* track; no villain/wizard gameplay use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="77" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B17" s="78" t="str">
+        <x:v>intro_mild</x:v>
+      </x:c>
+      <x:c r="C17" s="78" t="str"/>
+      <x:c r="D17" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="78" t="str">
+        <x:v>Protected intro_* track; no villain/wizard gameplay use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="77" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B18" s="78" t="str">
+        <x:v>loopy1</x:v>
+      </x:c>
+      <x:c r="C18" s="78" t="str"/>
+      <x:c r="D18" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="78" t="str">
+        <x:v>Protected loop* track; no villain/wizard gameplay use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="77" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B19" s="78" t="str">
+        <x:v>loopystart</x:v>
+      </x:c>
+      <x:c r="C19" s="78" t="str">
+        <x:v>All villain/wizard bookend intros</x:v>
+      </x:c>
+      <x:c r="D19" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="78" t="str">
+        <x:v>Protected loop* track retained only as shared transition/intro music, not gameplay.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="77" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B20" s="78" t="str">
+        <x:v>loop_123</x:v>
+      </x:c>
+      <x:c r="C20" s="78" t="str"/>
+      <x:c r="D20" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="78" t="str">
+        <x:v>Protected loop* track; no villain/wizard gameplay use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="77" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B21" s="78" t="str">
+        <x:v>loop_123456</x:v>
+      </x:c>
+      <x:c r="C21" s="78" t="str">
+        <x:v>Main play random pool</x:v>
+      </x:c>
+      <x:c r="D21" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E21" s="78" t="str">
+        <x:v>Protected loop* track retained outside villain/wizard gameplay.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="73" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B22" s="74" t="str">
+        <x:v>maintheme</x:v>
+      </x:c>
+      <x:c r="C22" s="74" t="str">
+        <x:v>Attract</x:v>
+      </x:c>
+      <x:c r="D22" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E22" s="74" t="str">
+        <x:v>Protected main theme retained outside villain/wizard gameplay.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="73" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B23" s="74" t="str">
+        <x:v>paroxism</x:v>
+      </x:c>
+      <x:c r="C23" s="74" t="str">
+        <x:v>Doctor Octopus</x:v>
+      </x:c>
+      <x:c r="D23" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E23" s="74" t="str"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="73" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B24" s="74" t="str">
+        <x:v>shakeandstone</x:v>
+      </x:c>
+      <x:c r="C24" s="74" t="str">
+        <x:v>Parafino; Vulcan</x:v>
+      </x:c>
+      <x:c r="D24" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E24" s="74" t="str"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="73" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B25" s="74" t="str">
+        <x:v>somethings_up</x:v>
+      </x:c>
+      <x:c r="C25" s="74" t="str">
+        <x:v>Chapter Select; Villain Select</x:v>
+      </x:c>
+      <x:c r="D25" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E25" s="74" t="str"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="73" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B26" s="74" t="str">
+        <x:v>spider_intro_strong</x:v>
+      </x:c>
+      <x:c r="C26" s="74" t="str">
+        <x:v>All villain/wizard bookend summaries</x:v>
+      </x:c>
+      <x:c r="D26" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="74" t="str">
+        <x:v>Shared summary context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="73" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B27" s="74" t="str">
+        <x:v>street_beat</x:v>
+      </x:c>
+      <x:c r="C27" s="74" t="str">
+        <x:v>Rhino Bash</x:v>
+      </x:c>
+      <x:c r="D27" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E27" s="74" t="str"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="73" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B28" s="74" t="str">
+        <x:v>tautwalk</x:v>
+      </x:c>
+      <x:c r="C28" s="74" t="str">
+        <x:v>Electro; Time Showdown</x:v>
+      </x:c>
+      <x:c r="D28" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E28" s="74" t="str"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="73" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B29" s="74" t="str">
+        <x:v>twilight_guitar</x:v>
+      </x:c>
+      <x:c r="C29" s="74" t="str">
+        <x:v>Mysterio; Infinata</x:v>
+      </x:c>
+      <x:c r="D29" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E29" s="74" t="str"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="73" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B30" s="74" t="str">
+        <x:v>waiting</x:v>
+      </x:c>
+      <x:c r="C30" s="74" t="str">
+        <x:v>Scorpion; 5th Ave Phantom</x:v>
+      </x:c>
+      <x:c r="D30" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E30" s="74" t="str"/>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="77" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B31" s="78" t="str">
+        <x:v>intro_mild</x:v>
+      </x:c>
+      <x:c r="C31" s="78" t="str"/>
+      <x:c r="D31" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="78" t="str">
+        <x:v>Protected intro_* duplicate; unused.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="73" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B32" s="74" t="str">
+        <x:v>dash_to_safety_2</x:v>
+      </x:c>
+      <x:c r="C32" s="74" t="str">
+        <x:v>Dr. Magneto; The Spider-Men</x:v>
+      </x:c>
+      <x:c r="D32" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E32" s="74" t="str"/>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="73" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B33" s="74" t="str">
+        <x:v>dash_to_safety_3</x:v>
+      </x:c>
+      <x:c r="C33" s="74" t="str">
+        <x:v>Professor Pretorius; Charles Cameo</x:v>
+      </x:c>
+      <x:c r="D33" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E33" s="74" t="str"/>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="73" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B34" s="74" t="str">
+        <x:v>anji</x:v>
+      </x:c>
+      <x:c r="C34" s="74" t="str">
+        <x:v>Cerberus</x:v>
+      </x:c>
+      <x:c r="D34" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E34" s="74" t="str"/>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="73" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B35" s="74" t="str">
+        <x:v>besame_mucho</x:v>
+      </x:c>
+      <x:c r="C35" s="74" t="str">
+        <x:v>Diana</x:v>
+      </x:c>
+      <x:c r="D35" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="74" t="str"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="73" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B36" s="74" t="str">
+        <x:v>blood_and_black_lace</x:v>
+      </x:c>
+      <x:c r="C36" s="74" t="str">
+        <x:v>Centaur Charge</x:v>
+      </x:c>
+      <x:c r="D36" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E36" s="74" t="str"/>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="73" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B37" s="74" t="str">
+        <x:v>danube_incident</x:v>
+      </x:c>
+      <x:c r="C37" s="74" t="str">
+        <x:v>The Fly Twins</x:v>
+      </x:c>
+      <x:c r="D37" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E37" s="74" t="str"/>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="73" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B38" s="74" t="str">
+        <x:v>happy_go_lively</x:v>
+      </x:c>
+      <x:c r="C38" s="74" t="str">
+        <x:v>The Enforcers</x:v>
+      </x:c>
+      <x:c r="D38" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E38" s="74" t="str"/>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="73" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B39" s="74" t="str">
+        <x:v>la_buritta</x:v>
+      </x:c>
+      <x:c r="C39" s="74" t="str">
+        <x:v>The Fantastic Fakir</x:v>
+      </x:c>
+      <x:c r="D39" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E39" s="74" t="str"/>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="73" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B40" s="74" t="str">
+        <x:v>spooky</x:v>
+      </x:c>
+      <x:c r="C40" s="74" t="str">
+        <x:v>Kotep; Super Swami</x:v>
+      </x:c>
+      <x:c r="D40" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E40" s="74" t="str"/>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="73" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B41" s="74" t="str">
+        <x:v>sunflower</x:v>
+      </x:c>
+      <x:c r="C41" s="74" t="str">
+        <x:v>Dr. Noah Boddy</x:v>
+      </x:c>
+      <x:c r="D41" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="74" t="str"/>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="73" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B42" s="74" t="str">
+        <x:v>the_enchanted_sea</x:v>
+      </x:c>
+      <x:c r="C42" s="74" t="str">
+        <x:v>Doctor Dumpty; Doctor Atlantean</x:v>
+      </x:c>
+      <x:c r="D42" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E42" s="74" t="str"/>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="73" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B43" s="74" t="str">
+        <x:v>the_hearse</x:v>
+      </x:c>
+      <x:c r="C43" s="74" t="str">
+        <x:v>Doctor Zapp; The Web Tightens</x:v>
+      </x:c>
+      <x:c r="D43" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E43" s="74" t="str"/>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="73" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B44" s="74" t="str">
+        <x:v>the_ox</x:v>
+      </x:c>
+      <x:c r="C44" s="74" t="str">
+        <x:v>The Snowman</x:v>
+      </x:c>
+      <x:c r="D44" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E44" s="74" t="str"/>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="73" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B45" s="74" t="str">
+        <x:v>yegelle_tezeta</x:v>
+      </x:c>
+      <x:c r="C45" s="74" t="str">
+        <x:v>Dr. Manta</x:v>
+      </x:c>
+      <x:c r="D45" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E45" s="74" t="str"/>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="73" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B46" s="74" t="str">
+        <x:v>action_line</x:v>
+      </x:c>
+      <x:c r="C46" s="74" t="str">
+        <x:v>Desperado; The Plotter</x:v>
+      </x:c>
+      <x:c r="D46" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E46" s="74" t="str"/>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="73" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B47" s="74" t="str">
+        <x:v>the_shadows</x:v>
+      </x:c>
+      <x:c r="C47" s="74" t="str">
+        <x:v>The Plutonians; The Molemen</x:v>
+      </x:c>
+      <x:c r="D47" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E47" s="74" t="str"/>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="73" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B48" s="74" t="str">
+        <x:v>fbi</x:v>
+      </x:c>
+      <x:c r="C48" s="74" t="str">
+        <x:v>Igor; Crime Wave</x:v>
+      </x:c>
+      <x:c r="D48" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E48" s="74" t="str"/>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="73" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B49" s="74" t="str">
+        <x:v>don_and_dewey</x:v>
+      </x:c>
+      <x:c r="C49" s="74" t="str">
+        <x:v>Conner's Reptiles; Nature Strikes Back</x:v>
+      </x:c>
+      <x:c r="D49" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E49" s="74" t="str"/>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="73" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B50" s="74" t="str">
+        <x:v>beat_girl</x:v>
+      </x:c>
+      <x:c r="C50" s="74" t="str">
+        <x:v>Master Technician</x:v>
+      </x:c>
+      <x:c r="D50" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E50" s="74" t="str"/>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="73" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B51" s="74" t="str">
+        <x:v>aztec</x:v>
+      </x:c>
+      <x:c r="C51" s="74" t="str">
+        <x:v>Baron Von Rantenraven</x:v>
+      </x:c>
+      <x:c r="D51" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E51" s="74" t="str"/>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="73" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B52" s="74" t="str">
+        <x:v>motorcycle_circus</x:v>
+      </x:c>
+      <x:c r="C52" s="74" t="str">
+        <x:v>Mastermind Trap; Trubble Unleashed</x:v>
+      </x:c>
+      <x:c r="D52" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E52" s="74" t="str"/>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="73" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B53" s="74" t="str">
+        <x:v>peace_pipe</x:v>
+      </x:c>
+      <x:c r="C53" s="74" t="str">
+        <x:v>Fifth Dimension Curse</x:v>
+      </x:c>
+      <x:c r="D53" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E53" s="74" t="str"/>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="73" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B54" s="74" t="str">
+        <x:v>tall_cool_one</x:v>
+      </x:c>
+      <x:c r="C54" s="74" t="str">
+        <x:v>Who Is the Real Villain?</x:v>
+      </x:c>
+      <x:c r="D54" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E54" s="74" t="str"/>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="73" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B55" s="74" t="str">
+        <x:v>clasical_gas</x:v>
+      </x:c>
+      <x:c r="C55" s="74" t="str">
+        <x:v>Fiddler; Sinister Surge</x:v>
+      </x:c>
+      <x:c r="D55" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E55" s="74" t="str"/>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="73" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B56" s="74" t="str">
+        <x:v>sleepwalk</x:v>
+      </x:c>
+      <x:c r="C56" s="74" t="str">
+        <x:v>Harley Clivendon</x:v>
+      </x:c>
+      <x:c r="D56" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E56" s="74" t="str"/>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="73" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B57" s="74" t="str">
+        <x:v>topsy</x:v>
+      </x:c>
+      <x:c r="C57" s="74" t="str">
+        <x:v>Devargas; Brutus</x:v>
+      </x:c>
+      <x:c r="D57" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E57" s="74" t="str"/>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="73" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B58" s="74" t="str">
+        <x:v>moon_godess</x:v>
+      </x:c>
+      <x:c r="C58" s="74" t="str">
+        <x:v>Pardo; Master Vine</x:v>
+      </x:c>
+      <x:c r="D58" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E58" s="74" t="str"/>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="73" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B59" s="74" t="str">
+        <x:v>conquistador</x:v>
+      </x:c>
+      <x:c r="C59" s="74" t="str">
+        <x:v>The Conquistador</x:v>
+      </x:c>
+      <x:c r="D59" s="73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E59" s="74" t="str"/>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="73" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B60" s="74" t="str">
+        <x:v>death_have_no_mercy</x:v>
+      </x:c>
+      <x:c r="C60" s="74" t="str">
+        <x:v>Spider-Slayer; Lost World Invasion</x:v>
+      </x:c>
+      <x:c r="D60" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E60" s="74" t="str">
+        <x:v>New track now integrated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="A61" s="73" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B61" s="74" t="str">
+        <x:v>diamond_head</x:v>
+      </x:c>
+      <x:c r="C61" s="74" t="str">
+        <x:v>Doctor Cool; Mad Science Meltdown</x:v>
+      </x:c>
+      <x:c r="D61" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E61" s="74" t="str">
+        <x:v>New track now integrated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="73" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B62" s="74" t="str">
+        <x:v>washington_square</x:v>
+      </x:c>
+      <x:c r="C62" s="74" t="str">
+        <x:v>Clive and Blotto; Sir Galahad</x:v>
+      </x:c>
+      <x:c r="D62" s="73" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E62" s="74" t="str">
+        <x:v>New track now integrated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="75" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B63" s="76" t="str">
+        <x:v>bongo_rock</x:v>
+      </x:c>
+      <x:c r="C63" s="76" t="str">
+        <x:v>Metal Monster; Bolton and Boomer</x:v>
+      </x:c>
+      <x:c r="D63" s="75" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E63" s="76" t="str">
+        <x:v>New track now integrated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="68" t="str">
+        <x:v>Wizard Music Source Audit</x:v>
+      </x:c>
+      <x:c r="B66" s="68"/>
+      <x:c r="C66" s="68"/>
+      <x:c r="D66" s="68"/>
+      <x:c r="E66" s="68"/>
+    </x:row>
+    <x:row r="67" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A67" s="80" t="str">
+        <x:v>Wizard</x:v>
+      </x:c>
+      <x:c r="B67" s="80" t="str">
+        <x:v>Canonical Song</x:v>
+      </x:c>
+      <x:c r="C67" s="80" t="str">
+        <x:v>Mode Config Override</x:v>
+      </x:c>
+      <x:c r="D67" s="80" t="str">
+        <x:v>Effective Song</x:v>
+      </x:c>
+      <x:c r="E67" s="80" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A68" s="14" t="str">
+        <x:v>Sinister Surge</x:v>
+      </x:c>
+      <x:c r="B68" s="14" t="str">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C68" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D68" s="14" t="str">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E68" s="14" t="str">
+        <x:v>Bookend assignment remains active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A69" s="14" t="str">
+        <x:v>Mastermind Trap</x:v>
+      </x:c>
+      <x:c r="B69" s="14" t="str">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C69" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D69" s="14" t="str">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="E69" s="14" t="str">
+        <x:v>Bookend assignment remains active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A70" s="14" t="str">
+        <x:v>Trubble Unleashed</x:v>
+      </x:c>
+      <x:c r="B70" s="14" t="str">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C70" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D70" s="14" t="str">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="E70" s="14" t="str">
+        <x:v>Bookend assignment remains active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A71" s="14" t="str">
+        <x:v>Fifth Dimension Curse</x:v>
+      </x:c>
+      <x:c r="B71" s="14" t="str">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C71" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D71" s="14" t="str">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="E71" s="14" t="str">
+        <x:v>Bookend assignment remains active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A72" s="14" t="str">
+        <x:v>Final Showdown / Kingpin</x:v>
+      </x:c>
+      <x:c r="B72" s="14" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C72" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D72" s="14" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E72" s="14" t="str">
+        <x:v>Bookend assignment remains active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="A74" s="68" t="str">
+        <x:v>Protected Track Family Audit</x:v>
+      </x:c>
+      <x:c r="B74" s="68"/>
+      <x:c r="C74" s="68"/>
+      <x:c r="D74" s="68"/>
+      <x:c r="E74" s="68"/>
+    </x:row>
+    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="A75" s="80" t="str">
+        <x:v>Family</x:v>
+      </x:c>
+      <x:c r="B75" s="80" t="str">
+        <x:v>Song / Asset</x:v>
+      </x:c>
+      <x:c r="C75" s="80" t="str">
+        <x:v>Villain/Wizard Gameplay</x:v>
+      </x:c>
+      <x:c r="D75" s="80" t="str">
+        <x:v>Flag</x:v>
+      </x:c>
+      <x:c r="E75" s="80" t="str">
+        <x:v>Allowed non-gameplay use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="A76" s="14" t="str">
+        <x:v>intro_*</x:v>
+      </x:c>
+      <x:c r="B76" s="14" t="str">
+        <x:v>11 — intro_loop_2</x:v>
+      </x:c>
+      <x:c r="C76" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D76" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E76" s="14" t="str">
+        <x:v>None currently</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="A77" s="14" t="str">
+        <x:v>intro_*</x:v>
+      </x:c>
+      <x:c r="B77" s="14" t="str">
+        <x:v>12 / 26 — intro_mild</x:v>
+      </x:c>
+      <x:c r="C77" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D77" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E77" s="14" t="str">
+        <x:v>None currently</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="A78" s="14" t="str">
+        <x:v>loop*</x:v>
+      </x:c>
+      <x:c r="B78" s="14" t="str">
+        <x:v>13 — loopy1</x:v>
+      </x:c>
+      <x:c r="C78" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D78" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E78" s="14" t="str">
+        <x:v>None currently</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="A79" s="14" t="str">
+        <x:v>loop*</x:v>
+      </x:c>
+      <x:c r="B79" s="14" t="str">
+        <x:v>14 — loopystart</x:v>
+      </x:c>
+      <x:c r="C79" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D79" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E79" s="14" t="str">
+        <x:v>Shared bookend intro transition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="A80" s="14" t="str">
+        <x:v>loop*</x:v>
+      </x:c>
+      <x:c r="B80" s="14" t="str">
+        <x:v>15 — loop_123</x:v>
+      </x:c>
+      <x:c r="C80" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D80" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E80" s="14" t="str">
+        <x:v>None currently</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="15" hidden="0" customHeight="1">
+      <x:c r="A81" s="14" t="str">
+        <x:v>loop*</x:v>
+      </x:c>
+      <x:c r="B81" s="14" t="str">
+        <x:v>16 — loop_123456</x:v>
+      </x:c>
+      <x:c r="C81" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D81" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E81" s="14" t="str">
+        <x:v>Main-play random pool</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="15" hidden="0" customHeight="1">
+      <x:c r="A82" s="14" t="str">
+        <x:v>maintheme</x:v>
+      </x:c>
+      <x:c r="B82" s="14" t="str">
+        <x:v>17 — maintheme</x:v>
+      </x:c>
+      <x:c r="C82" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D82" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="E82" s="14" t="str">
+        <x:v>Attract</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A3:E3"/>
+    <x:mergeCell ref="A66:E66"/>
+    <x:mergeCell ref="A74:E74"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -4873,10 +6183,10 @@
         <x:v>Doctor Zapp</x:v>
       </x:c>
       <x:c r="G38" s="31" t="str">
-        <x:v>Placeholder / design approved</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="H38" s="31" t="str">
-        <x:v>Knock down one target from each lower bank to open roof access. Upper spinner camera flashes defeat Zapp at 25 flashes; each lit upper helper target adds +1 flash per spin. Drops score 100K, helpers 50K, flashes 50K.</x:v>
+        <x:v>Camera Flash mode: qualify both lower banks, then use the rooftop spinner and unique upper-target boosts to reach 25 flashes. More Jackpots adds a 10-second bonus-spin window.</x:v>
       </x:c>
       <x:c r="I38" s="31" t="str">
         <x:v>nature_strikes_back</x:v>
@@ -4905,10 +6215,10 @@
         <x:v>Bolton and Boomer</x:v>
       </x:c>
       <x:c r="G39" s="31" t="str">
-        <x:v>Placeholder / design approved</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="H39" s="31" t="str">
-        <x:v>Repeating 2-ball multiball loop: hit a random lit target, lock one ball in any saucer, then shoot the VUK Super. First Super is untimed; later Supers run 20 seconds and reset the loop if missed.</x:v>
+        <x:v>Repeating 2-ball capture loop: hit a random lit target, lock one ball in any saucer, then shoot the VUK Super. The first Super is untimed; later Supers are timed.</x:v>
       </x:c>
       <x:c r="I39" s="31" t="str">
         <x:v>nature_strikes_back</x:v>
@@ -5001,10 +6311,10 @@
         <x:v>Dr. Manta</x:v>
       </x:c>
       <x:c r="G42" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="H42" s="31" t="str">
-        <x:v>Phantom from the Depths of Time villain. Dr. Manta rules the hidden city and ...</x:v>
+        <x:v>VUK-to-saucer relay: hold Ball 1 in the VUK, serve Ball 2 with a 10-second save, then lock it in any saucer. Kick Ball 1 to the rooftop for a 20-second attack. Either spinner raises the 100K jackpot by 50K per spin to a 1M cap; upper targets collect without resetting. At timeout all flippers disable until the active ball reaches the trough, then the held saucer ball is released.</x:v>
       </x:c>
       <x:c r="I42" s="31" t="str">
         <x:v>invasion_from_everywhere</x:v>
@@ -5129,10 +6439,10 @@
         <x:v>The Molemen</x:v>
       </x:c>
       <x:c r="G46" s="31" t="str">
-        <x:v>Placeholder/simple active mode</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="H46" s="31" t="str">
-        <x:v>Underground-world mode associated with Mugs Reilly and the Molemen. Compact l...</x:v>
+        <x:v>Two-ball area-control multiball. Left pop lights Saucer 1, center web lights Saucer 2, and right pop lights Saucer 3. Lit saucers award 250K per ball in play, reset their area, and can award one add-a-ball per area. A 5-second one-ball grace delays mode end.</x:v>
       </x:c>
       <x:c r="I46" s="31" t="str">
         <x:v>invasion_from_everywhere</x:v>
@@ -7347,7 +8657,7 @@
         <x:v>Elemental Chaos</x:v>
       </x:c>
       <x:c r="C38" s="31" t="str">
-        <x:v>dr_zap</x:v>
+        <x:v>dr_zapp</x:v>
       </x:c>
       <x:c r="D38" s="31" t="str">
         <x:v>Doctor Zapp</x:v>
@@ -7356,16 +8666,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F38" s="31" t="str">
-        <x:v>Placeholder framework for electrical machine / timed with invention control, using Spinner + lit shots.</x:v>
+        <x:v>Knock down one target from each lower bank to open roof access. Upper-spinner flashes defeat Zapp, while unique upper targets increase the flashes awarded per spin.</x:v>
       </x:c>
       <x:c r="G38" s="31" t="str">
-        <x:v>Ends when sequence complete / timer / ball end.</x:v>
+        <x:v>Complete 25 camera flashes; otherwise stop at ball end.</x:v>
       </x:c>
       <x:c r="H38" s="31" t="str">
-        <x:v>Zapp/Super value. Overload timing.</x:v>
+        <x:v>Drops score 100K, upper helpers score 50K, and each flash scores 50K. More Jackpots adds a timed bonus-spin window after completion.</x:v>
       </x:c>
       <x:c r="I38" s="31" t="str">
-        <x:v>Placeholder widget and progression state are active; full episode-based rules and presentation remain to be designed.</x:v>
+        <x:v>Implemented with custom code, YAML, widget, lighting, status and summary variables; needs on-machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -7376,25 +8686,25 @@
         <x:v>Elemental Chaos</x:v>
       </x:c>
       <x:c r="C39" s="31" t="str">
-        <x:v>voltan_boomer</x:v>
+        <x:v>bolton_boomer</x:v>
       </x:c>
       <x:c r="D39" s="31" t="str">
-        <x:v>Voltan and Boomer</x:v>
+        <x:v>Bolton and Boomer</x:v>
       </x:c>
       <x:c r="E39" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F39" s="31" t="str">
-        <x:v>Placeholder framework for storm timing / robbery with thunder windows, using Storm shots + target groups.</x:v>
+        <x:v>Hit a random lit target, capture one ball in any saucer, then shoot the VUK Super. After the release, repeat the loop.</x:v>
       </x:c>
       <x:c r="G39" s="31" t="str">
-        <x:v>Ends when goals completed / ball end.</x:v>
+        <x:v>Complete the required Super sequence or end when multiball returns to one ball / ball end.</x:v>
       </x:c>
       <x:c r="H39" s="31" t="str">
-        <x:v>Thunder/robbery jackpots. Short storm windows.</x:v>
+        <x:v>The first VUK Super is persistent. Later Super opportunities are timed and reset the capture loop when missed.</x:v>
       </x:c>
       <x:c r="I39" s="31" t="str">
-        <x:v>Placeholder widget and progression state are active; full episode-based rules and presentation remain to be designed.</x:v>
+        <x:v>Implemented with custom code, YAML, widget, capture handling, status and summary variables; needs on-machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -7469,19 +8779,19 @@
         <x:v>Dr. Manta</x:v>
       </x:c>
       <x:c r="E42" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>2 staged / 1 active</x:v>
       </x:c>
       <x:c r="F42" s="31" t="str">
-        <x:v>Placeholder framework for hidden-city control with trap / freeze, using Saucers + robotic-creature shots.</x:v>
+        <x:v>Shoot the VUK for 100K to hold Ball 1 and serve Ball 2 with a 10-second save. Lock Ball 2 in any saucer for 150K; it remains held while Ball 1 is kicked to the rooftop.</x:v>
       </x:c>
       <x:c r="G42" s="31" t="str">
-        <x:v>Ends when goals or timer / ball end.</x:v>
+        <x:v>After the 20-second attack expires, all flippers disable. When the active ball reaches the trough, the mode ends, the saucer ball releases, and normal single-ball play resumes. Losing Ball 2 before a saucer lock also ends the mode and releases the VUK ball.</x:v>
       </x:c>
       <x:c r="H42" s="31" t="str">
-        <x:v>Frozen-city jackpots. Held ball / trap pressure.</x:v>
+        <x:v>Jackpot starts at 100K. Either spinner adds 50K per spin, capped at 1M. Any upper target collects the current value without resetting it. More Time = 28s; Safety Net = 25s save; Bigger = 150K VUK / 200K saucer / 200K starting JP; More Jackpots = 75K per spin; Shot Assist makes the upper target corresponding to the occupied saucer worth 3X once.</x:v>
       </x:c>
       <x:c r="I42" s="31" t="str">
-        <x:v>Placeholder widget and progression state are active; full episode-based rules and presentation remain to be designed.</x:v>
+        <x:v>Implemented with phase lighting, live timer/value/jackpot status, one-time mapped 3X indication, timeout blackout, and summary variables; needs on-machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -7582,22 +8892,22 @@
         <x:v>molemen</x:v>
       </x:c>
       <x:c r="D46" s="31" t="str">
-        <x:v>Molemen</x:v>
+        <x:v>The Molemen</x:v>
       </x:c>
       <x:c r="E46" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F46" s="31" t="str">
-        <x:v>Placeholder framework for underground invasion with area / survival, using Drops, tunnels, lower playfield.</x:v>
+        <x:v>Two-ball multiball. Left pop, center web and right pop independently light Saucer 1, 2 and 3. The rooftop gate remains closed.</x:v>
       </x:c>
       <x:c r="G46" s="31" t="str">
-        <x:v>Ends when goals or timer / ball end.</x:v>
+        <x:v>When play drops to one ball, a 5-second grace begins before the mode ends; More Time increases it to 10 seconds. Mode also stops at ball end.</x:v>
       </x:c>
       <x:c r="H46" s="31" t="str">
-        <x:v>Underground jackpots. Escalating underground pressure.</x:v>
+        <x:v>Pop hits score 50K and center web scores 100K. A lit saucer awards 250K multiplied by balls in play and resets that area. Each area can qualify add-a-ball once: 3 left-pop hits, 1 center-web hit, or 3 right-pop hits.</x:v>
       </x:c>
       <x:c r="I46" s="31" t="str">
-        <x:v>Placeholder widget and progression state are active; full episode-based rules and presentation remain to be designed.</x:v>
+        <x:v>Implemented with three mapped areas, saucer jackpot/add-a-ball shows, custom widget, Case Files, grace handling and summary variables; needs on-machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -8272,20 +9582,42 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
-        <x:v>Villain music transition-track cleanup</x:v>
+        <x:v>Villain/wizard music rebalance</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>Reassigned Trubble Unleashed to motorcycle_circus; Fifth Avenue Phantom to waiting; The Plotter to fbi; The Plutonians to the_shadows; Nature Strikes Back to don_and_dewey. Selection/intro/summary tracks remain unchanged.</x:v>
+        <x:v>Rebalanced all villain/wizard gameplay songs to a maximum of two uses. Removed maintheme / loop* / intro_* gameplay assignments. Songs 55-58 are integrated. Wizard mode-level play_song overrides were removed so villain_bookends.py is the canonical assignment source.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
         <x:v>Implemented - needs test</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="14"/>
-      <x:c r="B19" s="14"/>
-      <x:c r="C19" s="14"/>
-      <x:c r="D19" s="14"/>
+      <x:c r="A19" s="14" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>Playtest Dr. Manta relay</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>Verify VUK hold, second-ball serve/save, saucer hold, VUK rooftop eject, both spinner increments, mapped one-time 3X target, all-flipper timeout, trough handoff, saucer release, and early second-ball-loss cleanup.</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Implemented - needs test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Playtest The Molemen</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Verify two-ball start, closed rooftop gate, three area-to-saucer mappings, per-ball jackpot values, one-use add-a-ball per area, saucer reset/eject timing, one-ball grace, Case Files, widget and cleanup.</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Implemented - needs test</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -8322,10 +9654,10 @@
         <x:v>Current full codebase</x:v>
       </x:c>
       <x:c r="B2" s="31" t="str">
-        <x:v>/mnt/data/ASM67_2026_07_24_3pm.zip</x:v>
+        <x:v>ASM67_2026_08_06_1am.zip</x:v>
       </x:c>
       <x:c r="C2" s="31" t="str">
-        <x:v>Current source-of-truth full ZIP supplied by the user.</x:v>
+        <x:v>Source-of-truth full ZIP supplied by the user; music rebalance applied 2026-08-06.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>

<commit_message>
cleanup and surge work
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8681d20a12c54d9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R1f64d79bd9344cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rdd10dcc57a9e44fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R77881bc7750e40be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rb017133334ef40e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Raafefa16eefb4d4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R62ea8e3523a5400a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R9891d68e1da54bcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rd8727351b67448d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R1b900bb4a95242c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rd21a5303022146d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R7c0f7bc9041e4ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R29a08e63619a4995"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4c38b157dbf146fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R783292e8935a4290"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R5f0d583591da4774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rddc19c9a102142a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R745bffc6793742c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R0caf176a8bfd4dee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R9c19d7245b484241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R910d30c9a6c54d98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rf34fad48a17649f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rfd802361e734457b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rbca53a62db924596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R4bbfadff598e42a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Reaab671bc7dc43ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -708,6 +708,17 @@
         <x:v>Former Kingpin limited-shot right-bank pursuit has been converted to Desperado without restoring the old Kingpin player-variable payload.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A12" s="14" t="str">
+        <x:v>Player-var cleanup</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>August 8 batch reduces declared player vars from 356 to 292 and moves temporary runtime state for seven modes into Python. Bookend summary contracts were corrected at the same time.</x:v>
+      </x:c>
+      <x:c r="C12" s="14"/>
+      <x:c r="D12" s="14"/>
+      <x:c r="E12" s="14"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -3024,8 +3035,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="68" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="59" t="str">
         <x:v>Area</x:v>
       </x:c>
@@ -3061,7 +3078,7 @@
       <x:c r="Y1" s="56"/>
       <x:c r="Z1" s="56"/>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="31" t="str">
         <x:v>Danger Lurks villains</x:v>
       </x:c>
@@ -3097,7 +3114,7 @@
       <x:c r="Y2" s="14"/>
       <x:c r="Z2" s="14"/>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="31" t="str">
         <x:v>The Web Tightens</x:v>
       </x:c>
@@ -3133,7 +3150,7 @@
       <x:c r="Y3" s="14"/>
       <x:c r="Z3" s="14"/>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="31" t="str">
         <x:v>The Web Tightens</x:v>
       </x:c>
@@ -3169,7 +3186,7 @@
       <x:c r="Y4" s="14"/>
       <x:c r="Z4" s="14"/>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="31" t="str">
         <x:v>Chapter 11 selection</x:v>
       </x:c>
@@ -3205,7 +3222,7 @@
       <x:c r="Y5" s="14"/>
       <x:c r="Z5" s="14"/>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="31" t="str">
         <x:v>Fiddler bonus</x:v>
       </x:c>
@@ -3219,7 +3236,7 @@
         <x:v>Persistent end-of-ball Chapter 5 bonus bank.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="31" t="str">
         <x:v>Crime Wave</x:v>
       </x:c>
@@ -3233,7 +3250,7 @@
         <x:v>Only persistent state required for the Chapter 4 wizard.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="31" t="str">
         <x:v>Crime Wave legacy</x:v>
       </x:c>
@@ -3247,7 +3264,7 @@
         <x:v>Obsolete predecessor variables; no active code or widget uses them.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="31" t="str">
         <x:v>Kingpin regular mode</x:v>
       </x:c>
@@ -3261,7 +3278,7 @@
         <x:v>Kingpin is now the final wizard identity; the old regular mode is unloaded and removed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="31" t="str">
         <x:v>Stale modes</x:v>
       </x:c>
@@ -3275,7 +3292,7 @@
         <x:v>Replaced by final_showdown/Kingpin and skymaster respectively.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="31" t="str">
         <x:v>Stale widgets</x:v>
       </x:c>
@@ -3289,7 +3306,7 @@
         <x:v>No active config references these widgets.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A12" s="14" t="str">
         <x:v>Desperado repurpose</x:v>
       </x:c>
@@ -3301,6 +3318,132 @@
       </x:c>
       <x:c r="D12" s="14" t="str">
         <x:v>Former Kingpin round, timer, target, and extra-round variables remain Python-only and are not exported to Godot.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="14" t="str">
+        <x:v>August 8 cleanup batch</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>config/player_vars.yaml: 356 -&gt; 292 declarations</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Net removal of 64 declarations; temporary mode-run state moved to Python while durable progression and shared summary data remain player state.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="14" t="str">
+        <x:v>Sinister Surge</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>Mode-local</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>~24 sinister_surge_* working/case-file variables</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Area progress, A/B, lit/ready flags, values and target counters now live in the mode runtime dictionary; *_state and shared summary counters persist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="14" t="str">
+        <x:v>Final Showdown</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>Mode-local</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>final_showdown_* live area/shot/jackpot working state</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Working state now lives in the mode runtime dictionary; only final_showdown_state plus shared summary counters persist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A16" s="14" t="str">
+        <x:v>Fly Twins</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>Mode-local</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>15 temporary fly_twins_* declarations removed</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Round telemetry, lit saucers, multiplier, spinner/target state and Shot Assist are Python-local. Only state plus two bookend stats remain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="14" t="str">
+        <x:v>Molemen</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>Mode-local</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>13 temporary molemen_* declarations removed</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Area hits/lights/add-a-ball readiness are held in a local area_state structure. Opening ball-save timing stays a player variable because MPF YAML reads it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="14" t="str">
+        <x:v>Trubble Unleashed</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>Mode-local</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>7 temporary trubble_unleashed_* declarations removed</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>Timer, staged targets, add-a-ball readiness, lit saucers and live value stay on the mode; only two bookend stats and progression/shared vars persist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="14" t="str">
+        <x:v>Dr. Manta</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>Mode-local</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>7 temporary dr_manta_* declarations removed</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>Phase, timer, held saucer, jackpot and Shot Assist telemetry are Python-local. Second-ball-save seconds remains for the current_player YAML timing expression.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="14" t="str">
+        <x:v>Fifth Avenue Phantom</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>Mode-local</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>Stopped dynamic creation of phase/location/timer/reveal/Shot Assist vars</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>Runtime telemetry remains on the Python mode. Only progression and the two explicit summary stats are player variables.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>Bookend summary contracts</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>Diana, Mysterio, Fly Twins, Super Swami, Sinister Surge, Trubble Unleashed, Fifth Dimension Curse, Final Showdown</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="str">
+        <x:v>Removed references to missing or incorrect summary variables; summaries now read counters that the corresponding gameplay modes actually populate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3350,7 +3493,7 @@
       <x:c r="Y1" s="56"/>
       <x:c r="Z1" s="56"/>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A2" s="31" t="str">
         <x:v>Classic Rogues</x:v>
       </x:c>
@@ -3364,7 +3507,7 @@
         <x:v>Sinister Surge</x:v>
       </x:c>
       <x:c r="E2" s="31" t="str">
-        <x:v>Implemented / needs playtest</x:v>
+        <x:v>Coded / needs machine playtest</x:v>
       </x:c>
       <x:c r="F2" s="14"/>
       <x:c r="G2" s="14"/>
@@ -6820,7 +6963,7 @@
         <x:v>Implementation Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A2" s="31" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -6840,7 +6983,7 @@
         <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G2" s="31" t="str">
-        <x:v>Implemented; needs continued playtest/polish.</x:v>
+        <x:v>Coded; needs on-machine playtest. Chapter 1 callbacks: Rhino 6 pops; Sandman flashing right-bank drop moves every 4s; Vulture 1 upper target + 3 upper-spinner spins in any order; Electro both webs with 20s for the second shot and reset on timeout; Green Goblin any saucer holds 4s, then hit 2 of 4 areas (left web, center web, left bank, right bank; any drop counts its bank). One ball may rest in a saucer for 20s outside Goblin. Existing stage Jackpot, A+B add-a-ball, and Victory Laps structure retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9616,6 +9759,20 @@
         <x:v>Verify two-ball start, closed rooftop gate, three area-to-saucer mappings, per-ball jackpot values, one-use add-a-ball per area, saucer reset/eject timing, one-ball grace, Case Files, widget and cleanup.</x:v>
       </x:c>
       <x:c r="D20" t="str">
+        <x:v>Implemented - needs test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>Playtest player-var cleanup batch</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>Regression-test Sinister Surge, Final Showdown, Fly Twins, Molemen, Fifth Avenue Phantom, Trubble Unleashed and Dr. Manta; verify end-of-mode summary stats after mode stop.</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="str">
         <x:v>Implemented - needs test</x:v>
       </x:c>
     </x:row>
@@ -9649,15 +9806,15 @@
         <x:v>Use</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="31" t="str">
         <x:v>Current full codebase</x:v>
       </x:c>
       <x:c r="B2" s="31" t="str">
-        <x:v>ASM67_2026_08_06_1am.zip</x:v>
+        <x:v>ASM67_2026_08_08_1pm.zip</x:v>
       </x:c>
       <x:c r="C2" s="31" t="str">
-        <x:v>Source-of-truth full ZIP supplied by the user; music rebalance applied 2026-08-06.</x:v>
+        <x:v>Source-of-truth full ZIP supplied by the user; August 8 player-variable cleanup applied to this baseline.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9735,6 +9892,17 @@
       </x:c>
       <x:c r="C9" s="14" t="str">
         <x:v>Case Files, progression, player variables, bookends, carousel mappings, and stale mode/widget assets audited against the 3pm baseline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="14" t="str">
+        <x:v>Player-variable cleanup</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>2026-08-08</x:v>
+      </x:c>
+      <x:c r="C10" s="14" t="str">
+        <x:v>Seven-mode runtime-state refactor plus villain_bookends summary-contract repair; declared player vars reduced from 356 to 292.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
lizard reviewed doc fixes
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4c38b157dbf146fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R783292e8935a4290"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R5f0d583591da4774"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rddc19c9a102142a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R745bffc6793742c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R0caf176a8bfd4dee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R9c19d7245b484241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R910d30c9a6c54d98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rf34fad48a17649f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rfd802361e734457b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rbca53a62db924596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R4bbfadff598e42a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Reaab671bc7dc43ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rca5e754bde204830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R117af33d254d41d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Ra940ec267d704892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R3e956232603e4ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rf7625bf8b37845cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R2154a5dd1f8b4363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R0a24d08e67884cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R8730d09b2ac243df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rc667405220c844a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R169e46b7324f47e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R75aeb8813f6c42af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R5082a3152e9b4c3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R1866e9dccf4744c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -636,12 +636,12 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A5" s="10" t="str">
         <x:v>Current focus</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>Danger Lurks is complete with five substantive villain modes. Elemental Chaos now has Clive and Blotto implemented, with Doctor Zapp, Bolton and Boomer, The Snowman, and The Plutonians designed but still awaiting implementation. Across all chapters, 40 of 55 regular villain modes have substantive implementations.</x:v>
+        <x:v>Danger Lurks is complete with five substantive villain modes. Elemental Chaos is also complete with five substantively coded villain modes; all five now need on-machine playtesting/polish. Across all chapters, 46 of 55 regular villain modes have substantive implementations.</x:v>
       </x:c>
       <x:c r="C5" s="14"/>
       <x:c r="D5" s="10" t="str">
@@ -707,17 +707,6 @@
       <x:c r="B11" s="14" t="str">
         <x:v>Former Kingpin limited-shot right-bank pursuit has been converted to Desperado without restoring the old Kingpin player-variable payload.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A12" s="14" t="str">
-        <x:v>Player-var cleanup</x:v>
-      </x:c>
-      <x:c r="B12" s="14" t="str">
-        <x:v>August 8 batch reduces declared player vars from 356 to 292 and moves temporary runtime state for seven modes into Python. Bookend summary contracts were corrected at the same time.</x:v>
-      </x:c>
-      <x:c r="C12" s="14"/>
-      <x:c r="D12" s="14"/>
-      <x:c r="E12" s="14"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3035,14 +3024,8 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="68" hidden="0" customWidth="1"/>
-  </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="1">
       <x:c r="A1" s="59" t="str">
         <x:v>Area</x:v>
       </x:c>
@@ -3078,7 +3061,7 @@
       <x:c r="Y1" s="56"/>
       <x:c r="Z1" s="56"/>
     </x:row>
-    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="2">
       <x:c r="A2" s="31" t="str">
         <x:v>Danger Lurks villains</x:v>
       </x:c>
@@ -3114,7 +3097,7 @@
       <x:c r="Y2" s="14"/>
       <x:c r="Z2" s="14"/>
     </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
+    <x:row r="3">
       <x:c r="A3" s="31" t="str">
         <x:v>The Web Tightens</x:v>
       </x:c>
@@ -3150,7 +3133,7 @@
       <x:c r="Y3" s="14"/>
       <x:c r="Z3" s="14"/>
     </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
+    <x:row r="4">
       <x:c r="A4" s="31" t="str">
         <x:v>The Web Tightens</x:v>
       </x:c>
@@ -3186,7 +3169,7 @@
       <x:c r="Y4" s="14"/>
       <x:c r="Z4" s="14"/>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5">
       <x:c r="A5" s="31" t="str">
         <x:v>Chapter 11 selection</x:v>
       </x:c>
@@ -3222,7 +3205,7 @@
       <x:c r="Y5" s="14"/>
       <x:c r="Z5" s="14"/>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6">
       <x:c r="A6" s="31" t="str">
         <x:v>Fiddler bonus</x:v>
       </x:c>
@@ -3236,7 +3219,7 @@
         <x:v>Persistent end-of-ball Chapter 5 bonus bank.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7">
       <x:c r="A7" s="31" t="str">
         <x:v>Crime Wave</x:v>
       </x:c>
@@ -3250,7 +3233,7 @@
         <x:v>Only persistent state required for the Chapter 4 wizard.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="8">
       <x:c r="A8" s="31" t="str">
         <x:v>Crime Wave legacy</x:v>
       </x:c>
@@ -3264,7 +3247,7 @@
         <x:v>Obsolete predecessor variables; no active code or widget uses them.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9">
       <x:c r="A9" s="31" t="str">
         <x:v>Kingpin regular mode</x:v>
       </x:c>
@@ -3278,7 +3261,7 @@
         <x:v>Kingpin is now the final wizard identity; the old regular mode is unloaded and removed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10">
       <x:c r="A10" s="31" t="str">
         <x:v>Stale modes</x:v>
       </x:c>
@@ -3292,7 +3275,7 @@
         <x:v>Replaced by final_showdown/Kingpin and skymaster respectively.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="11">
       <x:c r="A11" s="31" t="str">
         <x:v>Stale widgets</x:v>
       </x:c>
@@ -3306,7 +3289,7 @@
         <x:v>No active config references these widgets.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="12">
       <x:c r="A12" s="14" t="str">
         <x:v>Desperado repurpose</x:v>
       </x:c>
@@ -3318,132 +3301,6 @@
       </x:c>
       <x:c r="D12" s="14" t="str">
         <x:v>Former Kingpin round, timer, target, and extra-round variables remain Python-only and are not exported to Godot.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A13" s="14" t="str">
-        <x:v>August 8 cleanup batch</x:v>
-      </x:c>
-      <x:c r="B13" s="14" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="C13" s="14" t="str">
-        <x:v>config/player_vars.yaml: 356 -&gt; 292 declarations</x:v>
-      </x:c>
-      <x:c r="D13" s="14" t="str">
-        <x:v>Net removal of 64 declarations; temporary mode-run state moved to Python while durable progression and shared summary data remain player state.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A14" s="14" t="str">
-        <x:v>Sinister Surge</x:v>
-      </x:c>
-      <x:c r="B14" s="14" t="str">
-        <x:v>Mode-local</x:v>
-      </x:c>
-      <x:c r="C14" s="14" t="str">
-        <x:v>~24 sinister_surge_* working/case-file variables</x:v>
-      </x:c>
-      <x:c r="D14" s="14" t="str">
-        <x:v>Area progress, A/B, lit/ready flags, values and target counters now live in the mode runtime dictionary; *_state and shared summary counters persist.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A15" s="14" t="str">
-        <x:v>Final Showdown</x:v>
-      </x:c>
-      <x:c r="B15" s="14" t="str">
-        <x:v>Mode-local</x:v>
-      </x:c>
-      <x:c r="C15" s="14" t="str">
-        <x:v>final_showdown_* live area/shot/jackpot working state</x:v>
-      </x:c>
-      <x:c r="D15" s="14" t="str">
-        <x:v>Working state now lives in the mode runtime dictionary; only final_showdown_state plus shared summary counters persist.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A16" s="14" t="str">
-        <x:v>Fly Twins</x:v>
-      </x:c>
-      <x:c r="B16" s="14" t="str">
-        <x:v>Mode-local</x:v>
-      </x:c>
-      <x:c r="C16" s="14" t="str">
-        <x:v>15 temporary fly_twins_* declarations removed</x:v>
-      </x:c>
-      <x:c r="D16" s="14" t="str">
-        <x:v>Round telemetry, lit saucers, multiplier, spinner/target state and Shot Assist are Python-local. Only state plus two bookend stats remain.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A17" s="14" t="str">
-        <x:v>Molemen</x:v>
-      </x:c>
-      <x:c r="B17" s="14" t="str">
-        <x:v>Mode-local</x:v>
-      </x:c>
-      <x:c r="C17" s="14" t="str">
-        <x:v>13 temporary molemen_* declarations removed</x:v>
-      </x:c>
-      <x:c r="D17" s="14" t="str">
-        <x:v>Area hits/lights/add-a-ball readiness are held in a local area_state structure. Opening ball-save timing stays a player variable because MPF YAML reads it.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A18" s="14" t="str">
-        <x:v>Trubble Unleashed</x:v>
-      </x:c>
-      <x:c r="B18" s="14" t="str">
-        <x:v>Mode-local</x:v>
-      </x:c>
-      <x:c r="C18" s="14" t="str">
-        <x:v>7 temporary trubble_unleashed_* declarations removed</x:v>
-      </x:c>
-      <x:c r="D18" s="14" t="str">
-        <x:v>Timer, staged targets, add-a-ball readiness, lit saucers and live value stay on the mode; only two bookend stats and progression/shared vars persist.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A19" s="14" t="str">
-        <x:v>Dr. Manta</x:v>
-      </x:c>
-      <x:c r="B19" s="14" t="str">
-        <x:v>Mode-local</x:v>
-      </x:c>
-      <x:c r="C19" s="14" t="str">
-        <x:v>7 temporary dr_manta_* declarations removed</x:v>
-      </x:c>
-      <x:c r="D19" s="14" t="str">
-        <x:v>Phase, timer, held saucer, jackpot and Shot Assist telemetry are Python-local. Second-ball-save seconds remains for the current_player YAML timing expression.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A20" s="14" t="str">
-        <x:v>Fifth Avenue Phantom</x:v>
-      </x:c>
-      <x:c r="B20" s="14" t="str">
-        <x:v>Mode-local</x:v>
-      </x:c>
-      <x:c r="C20" s="14" t="str">
-        <x:v>Stopped dynamic creation of phase/location/timer/reveal/Shot Assist vars</x:v>
-      </x:c>
-      <x:c r="D20" s="14" t="str">
-        <x:v>Runtime telemetry remains on the Python mode. Only progression and the two explicit summary stats are player variables.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A21" s="14" t="str">
-        <x:v>Bookend summary contracts</x:v>
-      </x:c>
-      <x:c r="B21" s="14" t="str">
-        <x:v>Fixed</x:v>
-      </x:c>
-      <x:c r="C21" s="14" t="str">
-        <x:v>Diana, Mysterio, Fly Twins, Super Swami, Sinister Surge, Trubble Unleashed, Fifth Dimension Curse, Final Showdown</x:v>
-      </x:c>
-      <x:c r="D21" s="14" t="str">
-        <x:v>Removed references to missing or incorrect summary variables; summaries now read counters that the corresponding gameplay modes actually populate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3493,7 +3350,7 @@
       <x:c r="Y1" s="56"/>
       <x:c r="Z1" s="56"/>
     </x:row>
-    <x:row r="2" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="2">
       <x:c r="A2" s="31" t="str">
         <x:v>Classic Rogues</x:v>
       </x:c>
@@ -3507,7 +3364,7 @@
         <x:v>Sinister Surge</x:v>
       </x:c>
       <x:c r="E2" s="31" t="str">
-        <x:v>Coded / needs machine playtest</x:v>
+        <x:v>Implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F2" s="14"/>
       <x:c r="G2" s="14"/>
@@ -3917,7 +3774,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="67" t="str">
-        <x:v>Source of truth: ASM67_2026_08_06_1am plus this music patch. villain_bookends.py is canonical for villain/wizard gameplay music.</x:v>
+        <x:v>Source of truth: ASM67_2026_08_08_7pm. villain_bookends.py is canonical for villain/wizard gameplay music.</x:v>
       </x:c>
       <x:c r="B2" s="67"/>
       <x:c r="C2" s="67"/>
@@ -5433,7 +5290,7 @@
         <x:v>Implemented / needs playtest polish</x:v>
       </x:c>
       <x:c r="H10" s="31" t="str">
-        <x:v>Serum at STAR; deliver to web shots. Case files now enhance the loop: Bigger ...</x:v>
+        <x:v>Serum at STAR; deliver to left web. A/B flash yellow while available and go solid when collected; A+B during active serum adds 500K, restarts the timer, and plays a GI celebration. Successful delivery plays a 2-second white/green web-target show before the next serum (or More Jackpots follow-up) begins. Timer expiry fades GI to off over 2 seconds; the next serum or final completion waits until the fade finishes.</x:v>
       </x:c>
       <x:c r="I10" s="31" t="str">
         <x:v>mastermind_trap</x:v>
@@ -6963,7 +6820,7 @@
         <x:v>Implementation Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="2">
       <x:c r="A2" s="31" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -6983,7 +6840,7 @@
         <x:v>Every Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files, for a 0–500K bonus). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:v>
       </x:c>
       <x:c r="G2" s="31" t="str">
-        <x:v>Coded; needs on-machine playtest. Chapter 1 callbacks: Rhino 6 pops; Sandman flashing right-bank drop moves every 4s; Vulture 1 upper target + 3 upper-spinner spins in any order; Electro both webs with 20s for the second shot and reset on timeout; Green Goblin any saucer holds 4s, then hit 2 of 4 areas (left web, center web, left bank, right bank; any drop counts its bank). One ball may rest in a saucer for 20s outside Goblin. Existing stage Jackpot, A+B add-a-ball, and Victory Laps structure retained.</x:v>
+        <x:v>Implemented; needs continued playtest/polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -8003,7 +7860,7 @@
         <x:v>Ends when serum deliveries are completed; otherwise stops on ball end.</x:v>
       </x:c>
       <x:c r="H10" s="31" t="str">
-        <x:v>STAR creates serum; web shots deliver it. Case files add bigger value, slower decay, follow-up jackpots, one serum-save, and first-delivery flexibility.</x:v>
+        <x:v>STAR creates serum; left web delivers it. A+B adds 500,000 to an active serum and restarts the delivery timer; A/B inserts flash yellow while available, go solid yellow when collected, and completion plays a short GI celebration. Case files add bigger value, slower decay, follow-up jackpots, one serum-save, and Shot Assist delivery flexibility.</x:v>
       </x:c>
       <x:c r="I10" s="31" t="str">
         <x:v>Improved: live serum objective/delivery progress between countdowns.</x:v>
@@ -9504,7 +9361,7 @@
         <x:v>Playtest first 4 wizards</x:v>
       </x:c>
       <x:c r="C2" s="45" t="str">
-        <x:v>Sinister Surge, Mastermind Trap, Trubble Unleashed, The Plotter.</x:v>
+        <x:v>Sinister Surge, Mastermind Trap, Trubble Unleashed, Crime Wave.</x:v>
       </x:c>
       <x:c r="D2" s="45" t="str">
         <x:v>Open</x:v>
@@ -9588,7 +9445,7 @@
         <x:v>Visual polish / images</x:v>
       </x:c>
       <x:c r="C8" s="45" t="str">
-        <x:v>Replace placeholder villain/mode images and verify paths. The Plotter carousel currently reuses the former Kingpin image until dedicated art is supplied.</x:v>
+        <x:v>Replace placeholder villain/mode images and verify paths. Crime Wave carousel currently reuses the former Kingpin image until dedicated art is supplied.</x:v>
       </x:c>
       <x:c r="D8" s="45" t="str">
         <x:v>Open</x:v>
@@ -9759,20 +9616,6 @@
         <x:v>Verify two-ball start, closed rooftop gate, three area-to-saucer mappings, per-ball jackpot values, one-use add-a-ball per area, saucer reset/eject timing, one-ball grace, Case Files, widget and cleanup.</x:v>
       </x:c>
       <x:c r="D20" t="str">
-        <x:v>Implemented - needs test</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A21" s="14" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="B21" s="14" t="str">
-        <x:v>Playtest player-var cleanup batch</x:v>
-      </x:c>
-      <x:c r="C21" s="14" t="str">
-        <x:v>Regression-test Sinister Surge, Final Showdown, Fly Twins, Molemen, Fifth Avenue Phantom, Trubble Unleashed and Dr. Manta; verify end-of-mode summary stats after mode stop.</x:v>
-      </x:c>
-      <x:c r="D21" s="14" t="str">
         <x:v>Implemented - needs test</x:v>
       </x:c>
     </x:row>
@@ -9806,15 +9649,15 @@
         <x:v>Use</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="2">
       <x:c r="A2" s="31" t="str">
         <x:v>Current full codebase</x:v>
       </x:c>
       <x:c r="B2" s="31" t="str">
-        <x:v>ASM67_2026_08_08_1pm.zip</x:v>
+        <x:v>ASM67_2026_08_08_7pm.zip</x:v>
       </x:c>
       <x:c r="C2" s="31" t="str">
-        <x:v>Source-of-truth full ZIP supplied by the user; August 8 player-variable cleanup applied to this baseline.</x:v>
+        <x:v>Current source-of-truth full ZIP supplied by the user; includes the music rebalance and subsequent August 8 work.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9892,17 +9735,6 @@
       </x:c>
       <x:c r="C9" s="14" t="str">
         <x:v>Case Files, progression, player variables, bookends, carousel mappings, and stale mode/widget assets audited against the 3pm baseline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A10" s="14" t="str">
-        <x:v>Player-variable cleanup</x:v>
-      </x:c>
-      <x:c r="B10" s="14" t="str">
-        <x:v>2026-08-08</x:v>
-      </x:c>
-      <x:c r="C10" s="14" t="str">
-        <x:v>Seven-mode runtime-state refactor plus villain_bookends summary-contract repair; declared player vars reduced from 356 to 292.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
vulcan, cerberus, cyclops clean up
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rca5e754bde204830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R117af33d254d41d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Ra940ec267d704892"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R3e956232603e4ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rf7625bf8b37845cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R2154a5dd1f8b4363"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R0a24d08e67884cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R8730d09b2ac243df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rc667405220c844a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R169e46b7324f47e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R75aeb8813f6c42af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R5082a3152e9b4c3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R1866e9dccf4744c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9fa97cf385f84943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rd01de714164f49d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R91a919fd5b984ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R96421597f6124fb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R456997dd73b14d76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R57266ba5a25d4e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R8645733a76914854"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Re6c4aef855a5481a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R5cac0ed2416a4bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rcda42f69e0cb4ad3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R16eaeca5e33147b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R9bba26e56d174446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R7b2efa29bf404011"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1171,7 +1171,7 @@
         <x:v>Chapter 2 multiball role; area-control and lit-saucer add-a-ball give it a distinct identity.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="250.8000030517578" hidden="0" customHeight="1">
       <x:c r="A12" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -1185,7 +1185,7 @@
         <x:v>Cerberus</x:v>
       </x:c>
       <x:c r="E12" s="31" t="str">
-        <x:v>Implemented / needs playtest polish</x:v>
+        <x:v>Implemented / needs machine playtest</x:v>
       </x:c>
       <x:c r="F12" s="31" t="str">
         <x:v>1</x:v>
@@ -1200,19 +1200,19 @@
         <x:v>Upper targets + saucers</x:v>
       </x:c>
       <x:c r="J12" s="31" t="str">
-        <x:v>Matching saucer 2X jackpots</x:v>
+        <x:v>Matching saucer 3X jackpots; per-saucer retained repeat with More Jackpots</x:v>
       </x:c>
       <x:c r="K12" s="31" t="str">
-        <x:v>Timer expiry</x:v>
+        <x:v>16s timer after first jackpot; upper target/spinner/saucer resets</x:v>
       </x:c>
       <x:c r="L12" s="31" t="str">
-        <x:v>3 saucer JPs / timer / ball end</x:v>
+        <x:v>Timer expiry / ball end; 3 jackpots is display-only</x:v>
       </x:c>
       <x:c r="M12" s="31" t="str">
-        <x:v>Timer/matching role.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+        <x:v>Timed matching role. CERBERUS DEFEATED is a 2-second presentation after the third jackpot; progression only requires that the mode has been played.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="250.8000030517578" hidden="0" customHeight="1">
       <x:c r="A13" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -1226,31 +1226,31 @@
         <x:v>Vulcan</x:v>
       </x:c>
       <x:c r="E13" s="31" t="str">
-        <x:v>Implemented / needs playtest polish</x:v>
+        <x:v>Implemented / needs machine playtest</x:v>
       </x:c>
       <x:c r="F13" s="31" t="str">
-        <x:v>2-ball MB; add-a-ball to 3</x:v>
+        <x:v>2-ball MB; repeatable add-a-ball to 3</x:v>
       </x:c>
       <x:c r="G13" s="31" t="str">
         <x:v>Multiball</x:v>
       </x:c>
       <x:c r="H13" s="31" t="str">
-        <x:v>Spinner build</x:v>
+        <x:v>Drop-bank cash / roof reset</x:v>
       </x:c>
       <x:c r="I13" s="31" t="str">
-        <x:v>Spinner + right drops + upper targets</x:v>
+        <x:v>Right bank + upper entry/targets; left bank with More Jackpots</x:v>
       </x:c>
       <x:c r="J13" s="31" t="str">
-        <x:v>Built Vulcan JP / eruption bonus</x:v>
+        <x:v>100K/150K Jackpot; +25K per upper hit to 1M; full Jackpot banks to vulcan_bonus</x:v>
       </x:c>
       <x:c r="K13" s="31" t="str">
-        <x:v>MB drain + inactivity timeout</x:v>
+        <x:v>Multiball drain; exhausted banks wait for upper entry</x:v>
       </x:c>
       <x:c r="L13" s="31" t="str">
-        <x:v>MB/inactivity end</x:v>
+        <x:v>Multiball reaches 1 ball / ball end</x:v>
       </x:c>
       <x:c r="M13" s="31" t="str">
-        <x:v>Chapter MB role; strongly physical.</x:v>
+        <x:v>Chapter multiball role. Upper playfield replenishes the drop-bank cashout loop; repeatable Add-a-Ball rewards bank completion without a separate single-ball phase.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1294,7 +1294,7 @@
         <x:v>Limited-resource precision role with a clear red-GI Hunt state.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="316.79998779296875" hidden="0" customHeight="1">
       <x:c r="A15" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -1308,10 +1308,10 @@
         <x:v>Cyclops</x:v>
       </x:c>
       <x:c r="E15" s="31" t="str">
-        <x:v>Implemented / needs playtest polish</x:v>
+        <x:v>Implemented / needs machine playtest</x:v>
       </x:c>
       <x:c r="F15" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>1-ball limited flips; timed second Eye with More Jackpots</x:v>
       </x:c>
       <x:c r="G15" s="31" t="str">
         <x:v>Limited flips</x:v>
@@ -1320,19 +1320,19 @@
         <x:v>Build-to-cash</x:v>
       </x:c>
       <x:c r="I15" s="31" t="str">
-        <x:v>Drops + center web</x:v>
+        <x:v>Drops + rubbers + center web</x:v>
       </x:c>
       <x:c r="J15" s="31" t="str">
-        <x:v>Eye value from flips remaining</x:v>
+        <x:v>Eye = 100K x remaining flips (150K Bigger), cap 2M</x:v>
       </x:c>
       <x:c r="K15" s="31" t="str">
-        <x:v>Flip limit</x:v>
+        <x:v>Flip budget; second Eye has a 20s timer</x:v>
       </x:c>
       <x:c r="L15" s="31" t="str">
-        <x:v>Eye collected / flips out / ball end</x:v>
+        <x:v>Final Eye / flips out / second-Eye timeout / ball end</x:v>
       </x:c>
       <x:c r="M15" s="31" t="str">
-        <x:v>Limited-resource role.</x:v>
+        <x:v>Limited-resource role: drops (+3) and rubbers (+1) replenish an uncapped flip supply, but every flipper press spends one. More Jackpots converts the cashout into a second timed accuracy test.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -5331,7 +5331,7 @@
         <x:v>Mastermind Trap</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A12" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -5351,10 +5351,10 @@
         <x:v>Cerberus</x:v>
       </x:c>
       <x:c r="G12" s="31" t="str">
-        <x:v>Implemented / needs playtest polish</x:v>
+        <x:v>Implemented / needs machine playtest</x:v>
       </x:c>
       <x:c r="H12" s="31" t="str">
-        <x:v>Upper targets light saucers; matching saucer scores 2X; timer reset flow need...</x:v>
+        <x:v>Any upper target lights all saucers; its matching saucer is 3X. First jackpot starts the 16s timer; upper targets, upper spinner, and all saucer hits reset it. More Jackpots lets each saucer remain lit once after its first collection at the same state/multiplier. Shot Assist consumes one collection only. Third jackpot shows CERBERUS DEFEATED for 2s but play continues; playing the mode satisfies progression.</x:v>
       </x:c>
       <x:c r="I12" s="31" t="str">
         <x:v>trubble_unleashed</x:v>
@@ -5363,7 +5363,7 @@
         <x:v>Trubble Unleashed</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A13" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -5383,10 +5383,10 @@
         <x:v>Vulcan</x:v>
       </x:c>
       <x:c r="G13" s="31" t="str">
-        <x:v>Implemented / needs playtest polish</x:v>
+        <x:v>Implemented / needs machine playtest</x:v>
       </x:c>
       <x:c r="H13" s="31" t="str">
-        <x:v>Eruption multiball; spinner/right-drop scoring; upper set ramps vulcan_bonus.</x:v>
+        <x:v>2-ball Eruption multiball; right drops score a 100K Jackpot (150K Bigger) and upper-target hits add 25K to a 1M cap. Upper entry resets any down Jackpot banks. Bank completion qualifies repeatable Add-a-Ball at any upper target, capped at 3 balls. More Jackpots adds the left 3-bank. Upper-left exit holds the post 8s (12s More Time). Safety Net gives a 20s opening save; Shot Assist adds two right drops on the first right-drop hit. Every Jackpot adds its full value to vulcan_bonus.</x:v>
       </x:c>
       <x:c r="I13" s="31" t="str">
         <x:v>trubble_unleashed</x:v>
@@ -5427,7 +5427,7 @@
         <x:v>Trubble Unleashed</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A15" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -5447,10 +5447,10 @@
         <x:v>Cyclops</x:v>
       </x:c>
       <x:c r="G15" s="31" t="str">
-        <x:v>Implemented / needs playtest polish</x:v>
+        <x:v>Implemented / needs machine playtest</x:v>
       </x:c>
       <x:c r="H15" s="31" t="str">
-        <x:v>Limited flips; drops add flips; center-web Eye jackpot.</x:v>
+        <x:v>Limited flips: start 20 (30 More Time); drops add +3 and rubbers +1; banks reset immediately. Center-web Eye scores 100K x remaining flips (150K Bigger), capped at 2M. More Jackpots adds a second Eye after a 2s hold, then a 20s window; expiry shows EYE SEE YOU for 2s. Safety Net is a 10s ball save. Shot Assist makes the first drop hit knock down two additional right-bank targets, +3 flips each. Final Eye or 0 flips holds its message 2s before summary.</x:v>
       </x:c>
       <x:c r="I15" s="31" t="str">
         <x:v>trubble_unleashed</x:v>
@@ -7895,7 +7895,7 @@
         <x:v>Improved: persistent lit-saucer and collected-jackpot totals.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="541.2000122070312" hidden="0" customHeight="1">
       <x:c r="A12" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -7912,19 +7912,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F12" s="31" t="str">
-        <x:v>Upper targets light saucers; matching saucer collects stronger 2X jackpots while timer is active.</x:v>
+        <x:v>Hit upper targets to light all three saucers; the matching upper target makes its corresponding saucer a 3X jackpot. The upper spinner builds jackpot value.</x:v>
       </x:c>
       <x:c r="G12" s="31" t="str">
-        <x:v>Ends after 3 saucer jackpots, timer expiry, ball end, or mode completion state.</x:v>
+        <x:v>Timer expiry or ball end ends active play. Three jackpots only shows a 2-second CERBERUS DEFEATED message; it does not end the mode or gate progression.</x:v>
       </x:c>
       <x:c r="H12" s="31" t="str">
-        <x:v>Upper targets light saucers; matching saucer scores 2X; timer resets on key upper/spinner/saucer activity.</x:v>
+        <x:v>First jackpot starts a 16s timer (20s More Time). Upper targets, upper spinner, and any saucer hit reset it. After a collect the gate opens and other lit saucers return to 1X. More Jackpots gives each saucer one retained first collection at the same multiplier; Shot Assist is one use and consumes one collection on the awarded saucer.</x:v>
       </x:c>
       <x:c r="I12" s="31" t="str">
-        <x:v>Improved: persistent upper-target/saucer guidance and 3-jackpot progress.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+        <x:v>Reviewed/corrected; needs machine playtest. Orange GI retained; red saucer-hole and green 1/2/3 insert lighting remains lens-appropriate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="805.2000122070312" hidden="0" customHeight="1">
       <x:c r="A13" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -7938,19 +7938,19 @@
         <x:v>Vulcan</x:v>
       </x:c>
       <x:c r="E13" s="31" t="str">
-        <x:v>2-ball MB; add-a-ball to 3</x:v>
+        <x:v>2-ball MB; repeatable add-a-ball to 3</x:v>
       </x:c>
       <x:c r="F13" s="31" t="str">
-        <x:v>Eruption multiball: spinner builds Vulcan JP, right drops collect, upper target set can add a ball.</x:v>
+        <x:v>Start 2-ball multiball with the roof gate open. Right drops are Jackpots; upper targets build their value. Reaching the upper playfield resets any down targets in the active Jackpot banks.</x:v>
       </x:c>
       <x:c r="G13" s="31" t="str">
-        <x:v>Ends when down to 1 ball with no spinner activity for the timeout, or on ball end.</x:v>
+        <x:v>Ends when the main multiball reaches one ball, or on ball end. There is no Cooling Timer or single-ball continuation.</x:v>
       </x:c>
       <x:c r="H13" s="31" t="str">
-        <x:v>Eruption multiball; spinner builds Vulcan JP; right drops collect; upper target set can award add-a-ball/eruption bonus.</x:v>
+        <x:v>Jackpot starts 100K (150K Bigger), +25K per upper-target hit, capped at 1M. Completing an active bank qualifies one non-stacking Add-a-Ball; upper targets flash green until collected below the 3-ball cap. More Jackpots enables the left bank. Both banks reset only on upper entry. More Time makes the upper-left post hold 12s instead of 8s; Safety Net extends the opening save from 10s to 20s; Shot Assist awards two extra right drops on the first right-drop hit. Each Jackpot banks its full value to vulcan_bonus.</x:v>
       </x:c>
       <x:c r="I13" s="31" t="str">
-        <x:v>Good: active countdown/status and state-change messaging are present.</x:v>
+        <x:v>Reviewed/redesigned; needs machine playtest. Active bank GI pulses green and goes dark when exhausted; upper targets pulse purple normally and flash green for Add-a-Ball Ready.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -7982,7 +7982,7 @@
         <x:v>Arrows/time status, exit instruction, first-hit timer start, rubber arrow award, Hunt completion, and helper behavior are implemented.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="475.20001220703125" hidden="0" customHeight="1">
       <x:c r="A15" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -7996,19 +7996,19 @@
         <x:v>Cyclops</x:v>
       </x:c>
       <x:c r="E15" s="31" t="str">
-        <x:v>1</x:v>
+        <x:v>1-ball limited flips; timed second Eye with More Jackpots</x:v>
       </x:c>
       <x:c r="F15" s="31" t="str">
-        <x:v>Limited-flips mode: drops add flips, then center-web Eye collects based on remaining flips.</x:v>
+        <x:v>Start with 20 flips. Each flipper press spends 1; drops add 3; rubbers add 1; completed banks reset immediately. Center-web Eye is continuously indicated by a four-light white chase.</x:v>
       </x:c>
       <x:c r="G15" s="31" t="str">
-        <x:v>Ends when the Eye jackpot is collected, flips run out, or ball ends.</x:v>
+        <x:v>Ends after the final Eye Jackpot, at 0 flips, on second-Eye timeout, or on ball end. Final/failed presentations hold for 2s before summary.</x:v>
       </x:c>
       <x:c r="H15" s="31" t="str">
-        <x:v>Limited-flips mode; drop targets add flips; center-web Eye jackpot value depends on remaining flips.</x:v>
+        <x:v>Eye = remaining flips x 100K, cap 2M. Bigger = 150K x flips, same cap. More Time starts at 30 flips. More Jackpots: first Eye -&gt; 2s hold -&gt; second Eye for 20s, with no flip reset; drops/rubbers keep adding flips. Safety Net = 10s ball save. Shot Assist = first drop hit plus two additional right-bank drops, all worth +3 flips.</x:v>
       </x:c>
       <x:c r="I15" s="31" t="str">
-        <x:v>Good: flips-left status and state-change messaging are present.</x:v>
+        <x:v>Reviewed/redesigned; needs machine playtest. Overall GI D08080; both bank GI sections pulse purple. Eye chase: l_mid_multibonus -&gt; l_advance_multiplier -&gt; l_special -&gt; l_mid_web_target, white at 250ms per step.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -9824,7 +9824,7 @@
         <x:v>Implemented bank; carries over and is not multiplied by regular bonus X.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="31" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -9844,7 +9844,7 @@
         <x:v>VULCAN ERUPTION</x:v>
       </x:c>
       <x:c r="G4" s="31" t="str">
-        <x:v>Implemented bank; upper-target set starts at 75K and increases by 25K per completion.</x:v>
+        <x:v>Each collected Vulcan Jackpot adds its full scored value to the bank. Jackpot begins at 100K (150K with Bigger Jackpots), gains 25K per upper-target hit, and caps at 1M.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>

<commit_message>
reptiles and case file sfx
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcf7494480b8a4524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R4b21348701334b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R1e703278d3fb4319"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rafa75c4261bc4150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rfab60616bddf4323"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R5092dc63c08c40d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Re15b1cec6e754650"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rcbbf0e4f07f2457b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R0fd25d4d02bb4765"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Ra1372841388e4c20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R84d368b5d6664c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R3cac00ce6c604069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R79c7ed90cf67493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Refd875fe476f46bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rfa1a92083b4a4393"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R016ccd116ee4466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R209d2eb190054ba0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rfa24ec36404a44a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R1493e018d4664e27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R460f74445a17470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R540a8b6c70314d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rae39970a8be349f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Re65dd910f7214d0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R6e030d978f2e4293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R66caa01e10f1489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Rd50d5f4811694ddb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2784,31 +2784,31 @@
         <x:v>Conner's Reptiles</x:v>
       </x:c>
       <x:c r="E51" s="31" t="str">
-        <x:v>Implemented repurpose / needs polish</x:v>
+        <x:v>Redesigned / implemented / needs playtest</x:v>
       </x:c>
       <x:c r="F51" s="31" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G51" s="31" t="str">
-        <x:v>Banked bonus</x:v>
+        <x:v>Reveal-and-collect</x:v>
       </x:c>
       <x:c r="H51" s="31" t="str">
-        <x:v>Area hazard</x:v>
+        <x:v>Persistent bonus builder</x:v>
       </x:c>
       <x:c r="I51" s="31" t="str">
-        <x:v>Swamp shots</x:v>
+        <x:v>Pops + seven/eight revealed objectives + VUK</x:v>
       </x:c>
       <x:c r="J51" s="31" t="str">
-        <x:v>swamp_bonus bank</x:v>
+        <x:v>25K pops; +50K Swamp Bonus per counted pop; 100K/150K Jackpots; 500K Super</x:v>
       </x:c>
       <x:c r="K51" s="31" t="str">
-        <x:v>Escalating swamp pressure</x:v>
+        <x:v>Random unique objective reveals; gate held closed until final Super</x:v>
       </x:c>
       <x:c r="L51" s="31" t="str">
-        <x:v>Goals completed / ball end</x:v>
+        <x:v>All required Jackpots then VUK Super / ball end</x:v>
       </x:c>
       <x:c r="M51" s="31" t="str">
-        <x:v>Chapter bonus-bank/hazard role.</x:v>
+        <x:v>Distinct Chapter 10 bank-builder: pop action programs the playfield while all visible Jackpot shots remain available until collected.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -6606,10 +6606,10 @@
         <x:v>Conner's Reptiles</x:v>
       </x:c>
       <x:c r="G51" s="31" t="str">
-        <x:v>Implemented repurpose / needs polish</x:v>
+        <x:v>Redesigned / implemented / needs playtest</x:v>
       </x:c>
       <x:c r="H51" s="31" t="str">
-        <x:v>Repurposed Reptilla; real code retained under new name; swamp_bonus bank.</x:v>
+        <x:v>Swamp Rampage: every counted pop scores 25K, banks 50K Swamp Bonus, and reveals one unique random Jackpot from upper A/B, middle A/B, both webs, and grouped saucers. Collect all seven to open the gate for an untimed 500K VUK Super; More Jackpots adds the star.</x:v>
       </x:c>
       <x:c r="I51" s="31" t="str">
         <x:v>who_is_the_real_villain</x:v>
@@ -7143,7 +7143,7 @@
         <x:v>Conner's Reptiles</x:v>
       </x:c>
       <x:c r="D2" s="31" t="str">
-        <x:v>Reptilla code repurposed; active key is conners_reptiles.</x:v>
+        <x:v>Former Reptilla slot fully rewritten as Conner's Reptiles — Swamp Rampage.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9051,16 +9051,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F51" s="31" t="str">
-        <x:v>Play the retained Reptilla-style shot flow under the Swamp Reptiles identity.</x:v>
+        <x:v>Each counted pop scores 25K, adds 50K to persistent Swamp Bonus, and reveals one random unique Jackpot: upper A/B, middle A/B, left web, center web, or any saucer as one grouped objective. Pops continue adding bonus after all objectives are revealed.</x:v>
       </x:c>
       <x:c r="G51" s="31" t="str">
-        <x:v>Ends when retained Reptilla-style objectives complete; otherwise stops on ball end.</x:v>
+        <x:v>Collect all seven base Jackpots to open the rooftop gate and light the untimed VUK Super. More Jackpots adds the star as an eighth required objective. Only the collected VUK Super defeats the villain.</x:v>
       </x:c>
       <x:c r="H51" s="31" t="str">
-        <x:v>Repurposed Reptilla implementation; swamp_bonus bank preserved under new mode identity.</x:v>
+        <x:v>Jackpots 100K, or 150K with Bigger; VUK Super fixed at 500K. Safety Net 10s; More Time extends it to 20s. Shot Assist makes the first physical pop count twice: 50K score, +100K Swamp Bonus, and two Jackpots revealed.</x:v>
       </x:c>
       <x:c r="I51" s="31" t="str">
-        <x:v>Improved: persistent Rampage, lit-jackpot, collected-jackpot, and Super status.</x:v>
+        <x:v>Implemented rewrite. Starts in PLAYING state; only VUK Super collection posts completion. Gate is forced closed until Super, Daily Bugle VUK handling is suspended, lens-matched objective lamps pulse, and swamp_bonus is earned at 50K per counted pop.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -9465,13 +9465,13 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="B9" s="45" t="str">
-        <x:v>Light color cleanup</x:v>
+        <x:v>Playtest Conner's Reptiles / light color cleanup</x:v>
       </x:c>
       <x:c r="C9" s="45" t="str">
-        <x:v>Centaur, Diana, Enforcers, Conner's Reptiles; especially tinted right 5-bank/GI colors.</x:v>
+        <x:v>Verify random unique reveals; upper/middle A+B, both webs, grouped saucers and optional star; 25K pop scoring; +50K persistent Swamp Bonus per counted pop before/after Super; 100K/150K Jackpots; gate lockout; untimed 500K VUK Super; 10s/20s save; double-count Shot Assist; lens-matched pulsing; VUK summary hold and cleanup.</x:v>
       </x:c>
       <x:c r="D9" s="45" t="str">
-        <x:v>Open</x:v>
+        <x:v>Implemented - needs test</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -9549,10 +9549,10 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="B15" s="45" t="str">
-        <x:v>Chapter 5–11 bonus banks</x:v>
+        <x:v>Chapter 11 bonus bank</x:v>
       </x:c>
       <x:c r="C15" s="45" t="str">
-        <x:v>Harley Jackpots, Super Swami, Blotto Rampage, DeVargas Gold, and Invisible Fortune have earning rules. Implement the remaining later banks: swamp_bonus and technician_bonus.</x:v>
+        <x:v>swamp_bonus is implemented for Conner's Reptiles. Decide the Chapter 11 recipient and implement its remaining persistent bonus bank; technician_bonus remains the current placeholder.</x:v>
       </x:c>
       <x:c r="D15" s="45" t="str">
         <x:v>Future</x:v>
@@ -10081,10 +10081,10 @@
         <x:v>swamp_bonus</x:v>
       </x:c>
       <x:c r="F11" s="31" t="str">
-        <x:v>SWAMP REPTILES</x:v>
+        <x:v>SWAMP BONUS</x:v>
       </x:c>
       <x:c r="G11" s="31" t="str">
-        <x:v>Planned/declared Chapter 10 bank.</x:v>
+        <x:v>Implemented. Every counted pop scores 25K immediately and adds 50K to persistent swamp_bonus throughout the mode. Shot Assist makes the first physical pop count twice, adding 100K.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">

</xml_diff>

<commit_message>
fixes and more ab voices
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R678f3e591d6b46f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R662f1e9580614648"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R162c6f293cb040d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Raa050da44a5240c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R80ff688462a04754"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R443ce61fba524388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rbde67bf1cb0b4073"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rbbc6ed8c953e4d88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R16e2a63bea584cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R64a8ed2a24184204"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R88a72cbe4df14f6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Re40111ad9e1943b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R378c1d334cbe46c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R67bddbb232ae47d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R4877a3ed90b3405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R70c3d19dcd3a43ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R2d43fb56f43b49e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Rf209a773235a4f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R3c133828b3ae4f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rb8cb30a995964527"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R02d8507935694bc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R63ede562e9cc43e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rf4e244e4c0bb456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R4e385c76c86140fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R2facd949fec84729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R496c4833f7da46bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2490,10 +2490,8 @@
           <x:t xml:space="preserve">Fiddler</x:t>
         </x:is>
       </x:c>
-      <x:c r="E26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest</x:t>
-        </x:is>
+      <x:c r="E26" s="31" t="str">
+        <x:v>Implemented / recent retry-rule fix</x:v>
       </x:c>
       <x:c r="F26" s="31" t="inlineStr">
         <x:is>
@@ -2520,15 +2518,11 @@
           <x:t xml:space="preserve">Incrementing correct-note jackpots</x:t>
         </x:is>
       </x:c>
-      <x:c r="K26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Instant failure on wrong note</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3 rounds / optional 4th / wrong note / ball end</x:t>
-        </x:is>
+      <x:c r="K26" s="31" t="str">
+        <x:v>Startup and demonstration input lock prevents drop-knockdown vibration or live-ball switches from being judged before the response phase. Three mistakes are allowed per mode.</x:v>
+      </x:c>
+      <x:c r="L26" s="31" t="str">
+        <x:v>Complete Round 3 (or Round 4 with More Jackpots), or escape on the third mistake</x:v>
       </x:c>
       <x:c r="M26" s="31" t="inlineStr">
         <x:is>
@@ -3774,50 +3768,32 @@
           <x:t xml:space="preserve">The Molemen</x:t>
         </x:is>
       </x:c>
-      <x:c r="E46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Area-control multiball</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Saucer jackpots / add-a-ball</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Left pop, center web, right pop + three saucers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50K pops; 100K center; 250K per ball saucer jackpots</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Jackpot value depends on balls in play; each area offers one add-a-ball; short one-ball grace</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">One-ball grace expires / ball end</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chapter 9's conventional area-control multiball. It contrasts with Dr. Manta's staged relay, where one ball is always deliberately held.</x:t>
-        </x:is>
+      <x:c r="E46" s="31" t="str">
+        <x:v>Implemented / recent rule-device fix</x:v>
+      </x:c>
+      <x:c r="F46" s="31" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G46" s="31" t="str">
+        <x:v>Area-control multiball</x:v>
+      </x:c>
+      <x:c r="H46" s="31" t="str">
+        <x:v>Saucer jackpots / add-a-ball</x:v>
+      </x:c>
+      <x:c r="I46" s="31" t="str">
+        <x:v>Left pop, center web, right pop + three saucers</x:v>
+      </x:c>
+      <x:c r="J46" s="31" t="str">
+        <x:v>50K pops; 100K center; 250K per ball saucer jackpots</x:v>
+      </x:c>
+      <x:c r="K46" s="31" t="str">
+        <x:v>Jackpot value depends on balls in play; each area offers one add-a-ball with a 10-second shoot-again save, or 15 seconds with More Time</x:v>
+      </x:c>
+      <x:c r="L46" s="31" t="str">
+        <x:v>Molemen multiball ends / ball end</x:v>
+      </x:c>
+      <x:c r="M46" s="31" t="str">
+        <x:v>Chapter 9's conventional area-control multiball. It ends with the multiball device rather than offering an ineffective one-ball grace.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -4294,50 +4270,32 @@
           <x:t xml:space="preserve">Master Technician</x:t>
         </x:is>
       </x:c>
-      <x:c r="E54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Coded / needs machine test</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Timed score attack</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Risk/reward spinner build</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Drops + spinner + inlanes</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Each down target raises spinner value; stop at seven and spin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The eighth target costs 10 seconds and resets both banks</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">60-second timer expires / ball end</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Meteor-style spinner build retained in a repeatable 60-second loop; all five Case Files are implemented.</x:t>
-        </x:is>
+      <x:c r="E54" s="31" t="str">
+        <x:v>Implemented / recent widget-device-lighting fix</x:v>
+      </x:c>
+      <x:c r="F54" s="31" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G54" s="31" t="str">
+        <x:v>Timed score attack</x:v>
+      </x:c>
+      <x:c r="H54" s="31" t="str">
+        <x:v>Risk/reward spinner build</x:v>
+      </x:c>
+      <x:c r="I54" s="31" t="str">
+        <x:v>Drops + spinner + inlanes</x:v>
+      </x:c>
+      <x:c r="J54" s="31" t="str">
+        <x:v>25K drops; 10K unlit spinner; repeatable 50K per down target through seven</x:v>
+      </x:c>
+      <x:c r="K54" s="31" t="str">
+        <x:v>Building seven consumes much of the timer; the earned high spinner value remains repeatable. The eighth target costs 10 seconds and resets both banks.</x:v>
+      </x:c>
+      <x:c r="L54" s="31" t="str">
+        <x:v>60-second timer expires / ball end</x:v>
+      </x:c>
+      <x:c r="M54" s="31" t="str">
+        <x:v>Meteor-style spinner build retained with corrected portrait widget, closed lower-playfield route, staggered bank resets, and defined lens-safe lighting feedback.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -8221,15 +8179,11 @@
           <x:t xml:space="preserve">Fiddler</x:t>
         </x:is>
       </x:c>
-      <x:c r="G26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Simon Says violin mode. Three normal rounds use one, two, and three unique notes; More Jackpots adds a four-note round. Each note flashes for 2 seconds with a fixed audio event, then stays solid for ordered player input. One wrong note ends the mode.</x:t>
-        </x:is>
+      <x:c r="G26" s="31" t="str">
+        <x:v>Implemented / recent retry-rule fix</x:v>
+      </x:c>
+      <x:c r="H26" s="31" t="str">
+        <x:v>Simon Says violin mode. Three normal rounds use one, two, and three unique notes; More Jackpots adds a four-note encore. Each note flashes its ordered pulse pattern four times, then stays solid. Input is locked during startup drop knockdowns, setup delays, demonstrations, and replay delays. The first two mistakes restart the current round and replay the full pattern after 1.5s; the third mistake ends the mode. Shot Assist forgives the first wrong input without consuming a mistake.</x:v>
       </x:c>
       <x:c r="I26" s="31" t="inlineStr">
         <x:is>
@@ -9133,15 +9087,11 @@
           <x:t xml:space="preserve">The Molemen</x:t>
         </x:is>
       </x:c>
-      <x:c r="G46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Two-ball area-control multiball. Left pop lights Saucer 1, center web lights Saucer 2, and right pop lights Saucer 3. Lit saucers award 250K per ball in play, reset their area, and can award one add-a-ball per area. A 5-second one-ball grace delays mode end.</x:t>
-        </x:is>
+      <x:c r="G46" s="31" t="str">
+        <x:v>Implemented / recent rule-device fix</x:v>
+      </x:c>
+      <x:c r="H46" s="31" t="str">
+        <x:v>Two-ball area-control multiball. Left pop lights Saucer 1, center web lights Saucer 2, and right pop lights Saucer 3. Lit saucers award 250K per ball in play, reset their area, and can award one add-a-ball per area. The mode now ends immediately when multiball ends. More Time extends each add-a-ball shoot-again save from 10 to 15 seconds.</x:v>
       </x:c>
       <x:c r="I46" s="31" t="inlineStr">
         <x:is>
@@ -9501,15 +9451,11 @@
           <x:t xml:space="preserve">Master Technician</x:t>
         </x:is>
       </x:c>
-      <x:c r="G54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Coded / needs machine test</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">60-second spinner/drop score attack. Drops score 25K and build spinner value by 50K each through seven down; all eight costs 10 seconds and resets both banks. All five Case Files implemented.</x:t>
-        </x:is>
+      <x:c r="G54" s="31" t="str">
+        <x:v>Implemented / recent widget-device-lighting fix</x:v>
+      </x:c>
+      <x:c r="H54" s="31" t="str">
+        <x:v>60-second spinner/drop score attack. Drops score 25K and build a repeatable spinner value by 50K each through seven down; all eight costs 10 seconds and resets both banks. Widget now uses the existing portrait, the lower-playfield route closes the rooftop gate, bank resets are staggered 300ms, and complete lens-safe lighting/feedback is defined.</x:v>
       </x:c>
       <x:c r="I54" s="31" t="inlineStr">
         <x:is>
@@ -11976,25 +11922,17 @@
           <x:t xml:space="preserve">1</x:t>
         </x:is>
       </x:c>
-      <x:c r="F26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Watch a one-, two-, then three-note light-and-violin pattern using Left Web, Left Bank rubber, Center Web, and Right Bank rubber. Repeat each pattern in order.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Completes after Round 3, or Round 4 with More Jackpots. Any wrong note ends the mode unless the one-use Shot Assist awards the expected note.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Patterns demonstrate one light at a time. Its sequence-position pulse pattern repeats four times, then the light remains solid while the next note demonstrates. Positions 1-4 take 2.4s, 3.6s, 4.8s, and 6.0s. The pattern repeats after 14 seconds, or 8 with More Time. Correct-note scoring is 100K; 200K/300K; 400K/500K/600K; and 700K/800K/900K/1M in the optional fourth round. Bigger adds 100K to every note; Safety Net is the standard ball save.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I26" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented with fixed note events play_note_1 through play_note_4 mapped to violin_1 through violin_4, play_bad_note mapped to violin_bad_note, GI 60F060, and forced-down drop banks.</x:t>
-        </x:is>
+      <x:c r="F26" s="31" t="str">
+        <x:v>Watch each ordered violin pattern, then repeat it using Left Web, Left Bank rubber, Center Web, and Right Bank rubber.</x:v>
+      </x:c>
+      <x:c r="G26" s="31" t="str">
+        <x:v>Complete three rounds, or four with More Jackpots. Three mistakes during the mode allow Fiddler to escape.</x:v>
+      </x:c>
+      <x:c r="H26" s="31" t="str">
+        <x:v>Patterns contain one to four unique notes. Correct-note scoring remains 100K; 200K/300K; 400K/500K/600K; and 700K/800K/900K/1M in the optional encore.</x:v>
+      </x:c>
+      <x:c r="I26" s="31" t="str">
+        <x:v>Inputs are ignored until PLAY THE PATTERN. A non-terminal wrong note replays the complete current pattern after 1.5s. Shot Assist forgives the first wrong input and does not consume a mistake.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -12860,25 +12798,17 @@
           <x:t xml:space="preserve">2</x:t>
         </x:is>
       </x:c>
-      <x:c r="F46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Two-ball multiball. Left pop, center web and right pop independently light Saucer 1, 2 and 3. The rooftop gate remains closed.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">When play drops to one ball, a 5-second grace begins before the mode ends; More Time increases it to 10 seconds. Mode also stops at ball end.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pop hits score 50K and center web scores 100K. A lit saucer awards 250K multiplied by balls in play and resets that area. Each area can qualify add-a-ball once: 3 left-pop hits, 1 center-web hit, or 3 right-pop hits.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I46" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented with three mapped areas, saucer jackpot/add-a-ball shows, custom widget, Case Files, grace handling and summary variables; needs on-machine playtest.</x:t>
-        </x:is>
+      <x:c r="F46" s="31" t="str">
+        <x:v>Two-ball multiball. Left pop, center web and right pop independently light Saucer 1, 2 and 3. The rooftop gate remains closed.</x:v>
+      </x:c>
+      <x:c r="G46" s="31" t="str">
+        <x:v>The mode ends immediately when Molemen multiball ends. Mode also stops at ball end.</x:v>
+      </x:c>
+      <x:c r="H46" s="31" t="str">
+        <x:v>Pop hits score 50K and center web scores 100K. A lit saucer awards 250K multiplied by balls in play and resets that area. Each area can qualify add-a-ball once: 3 left-pop hits, 1 center-web hit, or 3 right-pop hits. More Time extends each add-a-ball shoot-again save from 10 to 15 seconds.</x:v>
+      </x:c>
+      <x:c r="I46" s="31" t="str">
+        <x:v>Implemented with three mapped areas, saucer jackpot/add-a-ball shows, corrected two-second saucer eject requests, immediate multiball-end handling, Case Files, status and summary variables; needs on-machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -13220,25 +13150,17 @@
           <x:t xml:space="preserve">1</x:t>
         </x:is>
       </x:c>
-      <x:c r="F54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">60-second spinner/drop score attack. Drops score 25K; spinner is 10K unlit and 50K per down target through seven. Inlanes knock down a standing target.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Timer expiry completes the mode; ball end stops it. All eight drops down deducts 10 seconds, resets both banks, and continues.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">More JP lights both web targets for 50K at levels 1-7; Bigger builds spinner at 75K per drop; More Time starts at 75s; Safety Net cancels first penalty; Shot Assist spots up to two safe targets.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I54" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Coded and documented; messages, seven-speed spinner/bank-GI pulses, summary stats, and player-var cleanup complete. Needs machine test.</x:t>
-        </x:is>
+      <x:c r="F54" s="31" t="str">
+        <x:v>60-second spinner/drop score attack. Drops score 25K; spinner is 10K unlit and 50K per down target through seven. Inlanes knock down a standing target. The built spinner value remains repeatable and does not reset on a spinner hit.</x:v>
+      </x:c>
+      <x:c r="G54" s="31" t="str">
+        <x:v>Timer expiry completes the mode; ball end stops it. All eight drops down deducts 10 seconds, resets both banks, and continues.</x:v>
+      </x:c>
+      <x:c r="H54" s="31" t="str">
+        <x:v>More JP lights both web targets for 50K at levels 1-7; Bigger builds spinner at 75K per drop; More Time starts at 75s; Safety Net cancels first penalty; Shot Assist spots up to two safe targets.</x:v>
+      </x:c>
+      <x:c r="I54" s="31" t="str">
+        <x:v>Implemented with portrait widget, closed rooftop gate, removed legacy upper-post action, 300ms bank-reset stagger, cool-blue base GI, seven-speed white spinner/bank pulses, drop/spinner feedback, short-circuit/Safety Net reactions, summary stats, and Case Files. Needs machine test.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -13607,10 +13529,8 @@
           <x:t xml:space="preserve">Cradle/status pages</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pages for goals, Chaos, photo/mystery, chapter/villain, extra balls, high-score context.</x:t>
-        </x:is>
+      <x:c r="C4" s="45" t="str">
+        <x:v>Shared persistent mode-status panel retained at 720 pixels to fit between the Player 3 and Player 4 score panels, with centered stacked title/value rows. Remaining pages for goals, Chaos, photo/mystery, chapter/villain, extra balls, and high-score context remain open.</x:v>
       </x:c>
       <x:c r="D4" s="45" t="inlineStr">
         <x:is>
@@ -13805,15 +13725,11 @@
           <x:t xml:space="preserve">Documentation</x:t>
         </x:is>
       </x:c>
-      <x:c r="C13" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roster, implementation status, wizard Case File rules, mode identities, and the Case File matrix are synced to code. No regular-villain Case File gaps remain. The loaded legacy daily_bugle_rooftop_riot placeholder is still documented. Master Technician, Sir Galahad, and Plotter need machine tests.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Updated 2026-08-17</x:t>
-        </x:is>
+      <x:c r="C13" s="45" t="str">
+        <x:v>Roster, implementation status, wizard Case File rules, mode identities, and the Case File matrix are synced to code. Master Technician's widget, gate, bank-reset and lighting fixes are documented; Master Technician, Sir Galahad, and Plotter still need machine tests.</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="str">
+        <x:v>Updated 2026-08-22</x:v>
       </x:c>
     </x:row>
     <x:row r="14" s="26" customFormat="1" ht="38" customHeight="1">
@@ -13959,10 +13875,8 @@
           <x:t xml:space="preserve">Playtest The Molemen</x:t>
         </x:is>
       </x:c>
-      <x:c r="C20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Verify two-ball start, closed rooftop gate, three area-to-saucer mappings, per-ball jackpot values, one-use add-a-ball per area, saucer reset/eject timing, one-ball grace, Case Files, widget and cleanup.</x:t>
-        </x:is>
+      <x:c r="C20" t="str">
+        <x:v>Verify two-ball start, closed rooftop gate, three area-to-saucer mappings, per-ball jackpot values, one-use add-a-ball per area, corrected two-second saucer eject timing, immediate mode end when multiball ends, 10s/15s add-a-ball shoot-again saves, Case Files, widget and cleanup.</x:v>
       </x:c>
       <x:c r="D20" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
vuk chase, fiddler and other things
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc5cb7bf8e9104e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R3239a4b192cb486a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R9720c182defc4071"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R6e700616d25c40d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R1ab261853aa64409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R500abf3dad224943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R9f0bd51e19e14d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R0dbc6b4d561b4760"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R65c7acabd1d14e15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rdcfd0d136d78488c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R52b11da9d41d4072"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R859e5932623f4f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R602813543d4e4d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfabe172fa1494ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R4b4c6a7b93184ebb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rf3671c9a8a524e16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Re2556a6421ae4781"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R595226a5a3124e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R693fbe008018486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R3c0512cb0e1746d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rdb573936551d4475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R94911920bf114b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rdfa5ed22392541ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R8f7e6639bbb54f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rcea3dcfaea5e40bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Re682346dab6c4412"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8591,7 +8591,7 @@
         <x:v>Implemented / recent spinner lighting fix</x:v>
       </x:c>
       <x:c r="H27" s="31" t="str">
-        <x:v>Five chances, or seven with More JP. Each chance presents three choices; spinner reveals the correct choice for 3s, or 5s with More Time. Three correct shots defeats Pardo immediately. Using all chances with fewer than three correct shots produces the escape result. Hidden choices use solid green for white/green lens compatibility; reveal flashes only the correct green choice and turns wrong choices off. The main spinner insert flashes white while choices are hidden, turns off during the reveal, and resumes if another reveal is needed. Result GI flashes for 350ms, then restores.</x:v>
+        <x:v>Five chances, or seven with More JP. Each chance presents three choices selected from seven logical shot groups; the three upper targets are one shared upper-target group so they can never show conflicting good/bad states. Spinner reveals the correct choice for 4s, or 6s with More Time. Three correct shots defeats Pardo immediately. Using all chances with fewer than three correct shots produces the escape result. Hidden choices use solid green for white/green lens compatibility; reveal flashes only the correct green choice and turns wrong choices off. The main spinner insert flashes white while choices are hidden, turns off during the reveal, and resumes if another reveal is needed. Result GI flashes for 350ms, then restores.</x:v>
       </x:c>
       <x:c r="I27" s="31" t="inlineStr">
         <x:is>
@@ -12198,10 +12198,10 @@
         <x:v>Third correct shot defeats Pardo; fewer than three correct after five chances (seven with More JP) lets him escape.</x:v>
       </x:c>
       <x:c r="H27" s="31" t="str">
-        <x:v>Spinner reveals the correct choice for 3 seconds (5 seconds with More Time). Correct Jackpots start at 100K and increase 50K; Bigger JP starts at 150K and increases 75K. Wrong choices score 10K and consume the chance.</x:v>
+        <x:v>Spinner reveals the correct choice for 4 seconds (6 seconds with More Time). Correct Jackpots start at 100K and increase 50K; Bigger JP starts at 150K and increases 75K. Wrong choices score 10K and consume the chance.</x:v>
       </x:c>
       <x:c r="I27" s="31" t="str">
-        <x:v>Nine possible shot groups; three are selected per chance. Hidden choices are solid green across white and green lenses. Reveal flashes only the correct choice green and turns wrong choices off. Result GI restores after a 350ms green/red confirmation. Shot Assist makes all three choices correct on the first chance. Summary outcome distinguishes defeat from escape.</x:v>
+        <x:v>Seven logical shot groups; three are selected per chance. Upper-left, upper-center, and upper-right targets are one grouped choice and always share the same good/bad state. Hidden choices are solid green across white and green lenses. Reveal flashes only the correct choice green and turns wrong choices off. Result GI restores after a 350ms green/red confirmation. Shot Assist makes all three choices correct on the first chance. Summary outcome distinguishes defeat from escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
more reviews and cleanup
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfabe172fa1494ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R4b4c6a7b93184ebb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rf3671c9a8a524e16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Re2556a6421ae4781"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R595226a5a3124e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R693fbe008018486a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R3c0512cb0e1746d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rdb573936551d4475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R94911920bf114b63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Rdfa5ed22392541ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R8f7e6639bbb54f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rcea3dcfaea5e40bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Re682346dab6c4412"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3313b8cce8b04e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Re8ed0d31a08f43b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R6a8c58c188964097"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R1b0956c0b3c144a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R233bc989fbc64ece"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Re2ba4c1aa4ea45ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Raa17dde6de784881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R425ad4d5b97943a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rebd86664dc724cc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R11e23c09aa034927"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R07e11370d2784538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R9bfbccb937ac4fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Ra81896037cee4cf2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2234,50 +2234,32 @@
           <x:t xml:space="preserve">Spider-Slayer</x:t>
         </x:is>
       </x:c>
-      <x:c r="E24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest polish</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expanding shot hunt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Persistent lit-shot growth</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ten lower-playfield categories + Daily Bugle VUK finish</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50K lit shots and a 2M decaying Slayer Jackpot</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fast 15-shot completion preserves more jackpot value</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Daily Bugle jackpot collected / ball end</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hunt Time measures first-to-fifteenth successful shot; jackpot value alone communicates the final urgency.</x:t>
-        </x:is>
+      <x:c r="E24" s="31" t="str">
+        <x:v>Implemented / reviewed; needs machine test</x:v>
+      </x:c>
+      <x:c r="F24" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G24" s="31" t="str">
+        <x:v>Expanding shot hunt</x:v>
+      </x:c>
+      <x:c r="H24" s="31" t="str">
+        <x:v>Persistent lit-shot growth with declining repeat values</x:v>
+      </x:c>
+      <x:c r="I24" s="31" t="str">
+        <x:v>Ten lower-playfield categories + Daily Bugle VUK finish</x:v>
+      </x:c>
+      <x:c r="J24" s="31" t="str">
+        <x:v>Per-category 50K/25K/10K/5K ladder; 2M timed Slayer Jackpot</x:v>
+      </x:c>
+      <x:c r="K24" s="31" t="str">
+        <x:v>15 hits open a 20-second VUK countdown; lit shots keep scoring</x:v>
+      </x:c>
+      <x:c r="L24" s="31" t="str">
+        <x:v>Jackpot collected / ball end; VUK opportunity expires and gate closes</x:v>
+      </x:c>
+      <x:c r="M24" s="31" t="str">
+        <x:v>Shot Assist counts/scores the first shot twice. All saucers share one counter and all six red hole lamps. Hunt Time is summarized only after 15 hits.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2299,50 +2281,32 @@
           <x:t xml:space="preserve">Metal-Eating Monster</x:t>
         </x:is>
       </x:c>
-      <x:c r="E25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Overlapping zone rescue</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Independent timers / escalating pressure</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Eight whole-playfield zones</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">250K zone saves; one half-value repeat per saved zone with More Jackpots</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">New attacks every 5s; saves accelerate the next attack to 2s</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4+ saved and no active attacks / 3 destroyed / ball end</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chapter 5 reversible-pressure role. Unlike Harley's accumulating area-control multiball, this is a single-ball rescue race with up to three overlapping independent deadlines.</x:t>
-        </x:is>
+      <x:c r="E25" s="31" t="str">
+        <x:v>Implemented / reviewed; saved-GI fix needs machine test</x:v>
+      </x:c>
+      <x:c r="F25" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G25" s="31" t="str">
+        <x:v>Overlapping zone rescue</x:v>
+      </x:c>
+      <x:c r="H25" s="31" t="str">
+        <x:v>Independent timers / escalating pressure</x:v>
+      </x:c>
+      <x:c r="I25" s="31" t="str">
+        <x:v>Eight whole-playfield zones</x:v>
+      </x:c>
+      <x:c r="J25" s="31" t="str">
+        <x:v>250K saves; one half-value saved-zone repeat with More Jackpots</x:v>
+      </x:c>
+      <x:c r="K25" s="31" t="str">
+        <x:v>New attacks every 5s; saves accelerate the next attack to 2s</x:v>
+      </x:c>
+      <x:c r="L25" s="31" t="str">
+        <x:v>Four saved and no active attacks / three destroyed / ball end</x:v>
+      </x:c>
+      <x:c r="M25" s="31" t="str">
+        <x:v>Attacks use 100% flashing orange GI plus native inserts. Saved zones remain visible with solid inserts and 75% green GI; destroyed zones are dark.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2480,50 +2444,32 @@
           <x:t xml:space="preserve">The Fantastic Fakir</x:t>
         </x:is>
       </x:c>
-      <x:c r="E28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / recent rule update</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2-ball MB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Multiball</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Saucer-to-roof</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Saucers + upper targets + spinners</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ruby JPs and Super</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MB drain / timing reveals</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MB end</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mystic chapter MB role.</x:t>
-        </x:is>
+      <x:c r="E28" s="31" t="str">
+        <x:v>Implemented / reviewed; VUK chase + status fix need machine test</x:v>
+      </x:c>
+      <x:c r="F28" s="31" t="str">
+        <x:v>2-ball MB</x:v>
+      </x:c>
+      <x:c r="G28" s="31" t="str">
+        <x:v>Multiball</x:v>
+      </x:c>
+      <x:c r="H28" s="31" t="str">
+        <x:v>Saucer-to-roof Ruby hunt</x:v>
+      </x:c>
+      <x:c r="I28" s="31" t="str">
+        <x:v>Saucers + VUK route + upper targets + both spinners</x:v>
+      </x:c>
+      <x:c r="J28" s="31" t="str">
+        <x:v>Ruby Jackpots and one summed Super</x:v>
+      </x:c>
+      <x:c r="K28" s="31" t="str">
+        <x:v>10s rooftop Ruby window; 15s with More Time</x:v>
+      </x:c>
+      <x:c r="L28" s="31" t="str">
+        <x:v>Multiball returns to one ball</x:v>
+      </x:c>
+      <x:c r="M28" s="31" t="str">
+        <x:v>Shared VUK chase stops on upper entry or attempt cleanup. Corrected status output uses real Ruby/Super state instead of nonexistent legacy flags.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2546,7 +2492,7 @@
         </x:is>
       </x:c>
       <x:c r="E29" s="31" t="str">
-        <x:v>Implemented / recent Scepter timer display fix</x:v>
+        <x:v>Implemented / reviewed; Scepter wording fix needs machine test</x:v>
       </x:c>
       <x:c r="F29" s="31" t="inlineStr">
         <x:is>
@@ -2578,7 +2524,7 @@
         <x:v>VUK Super or scepter timeout</x:v>
       </x:c>
       <x:c r="M29" s="31" t="str">
-        <x:v>Optional fifth demon with More Jackpots; persistent 20s/30s Scepter timer now shows the current VUK objective. Machine playtest pending.</x:v>
+        <x:v>Optional fifth demon with More Jackpots; persistent 20s/30s Scepter timer now directs SUPER AT DAILY BUGLE, or KILL THE DEMON, COLLECT THE SUPER while that demon remains. Machine playtest pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2601,7 +2547,7 @@
         </x:is>
       </x:c>
       <x:c r="E30" s="31" t="str">
-        <x:v>Implemented / recent failure-cleanup fix</x:v>
+        <x:v>Implemented / reviewed; flicker/status/gate fix needs machine test</x:v>
       </x:c>
       <x:c r="F30" s="31" t="inlineStr">
         <x:is>
@@ -2628,18 +2574,14 @@
           <x:t xml:space="preserve">Increasing restoration awards</x:t>
         </x:is>
       </x:c>
-      <x:c r="K30" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">40s blackout / 50s More Time</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L30" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Six restored / timer / ball end</x:t>
-        </x:is>
+      <x:c r="K30" s="31" t="str">
+        <x:v>Unrestored regions flicker independently for 100ms every random 2–5s; CITY TIME remains live through the Blackout finale.</x:v>
+      </x:c>
+      <x:c r="L30" s="31" t="str">
+        <x:v>Six restored / timer / ball end</x:v>
       </x:c>
       <x:c r="M30" s="31" t="str">
-        <x:v>Simple region-restoration role with optional VUK Blackout Jackpot. Timer failure now uses the centralized summary/cleanup pipeline; machine regression test pending.</x:v>
+        <x:v>More Jackpots adds the 500K Daily Bugle Blackout Jackpot. Its shared VUK chase starts after one guarded gate-open request. Timeout and success cleanup need machine regression testing.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2726,10 +2668,8 @@
           <x:t xml:space="preserve">Dr. Noah Boddy</x:t>
         </x:is>
       </x:c>
-      <x:c r="E32" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / recent rule update</x:t>
-        </x:is>
+      <x:c r="E32" s="31" t="str">
+        <x:v>Implemented / reviewed; lifecycle + VUK chase fix needs machine test</x:v>
       </x:c>
       <x:c r="F32" s="31" t="inlineStr">
         <x:is>
@@ -2756,20 +2696,14 @@
           <x:t xml:space="preserve">Secret-shot Jackpot plus uncapped upper-spinner build; each 25K/50K effective increment banks as INVISIBLE FORTUNE</x:t>
         </x:is>
       </x:c>
-      <x:c r="K32" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hidden info / wrong routing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L32" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Secret objectives solved / ball end</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M32" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mad Science reveal role.</x:t>
-        </x:is>
+      <x:c r="K32" s="31" t="str">
+        <x:v>Persistent cross-visit reveal state; shared VUK chase guides each rooftop return and one Python gate-open event owns access.</x:v>
+      </x:c>
+      <x:c r="L32" s="31" t="str">
+        <x:v>Secret objectives solved / hurry-up missed / ball end</x:v>
+      </x:c>
+      <x:c r="M32" s="31" t="str">
+        <x:v>Both success and missed/expired failure finish at completed state 2; their player-facing messages remain distinct. Machine regression testing pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2791,10 +2725,8 @@
           <x:t xml:space="preserve">Dr. Magneto</x:t>
         </x:is>
       </x:c>
-      <x:c r="E33" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented redesign / needs playtest</x:t>
-        </x:is>
+      <x:c r="E33" s="31" t="str">
+        <x:v>Implemented / reviewed; status + lighting fix needs machine test</x:v>
       </x:c>
       <x:c r="F33" s="31" t="inlineStr">
         <x:is>
@@ -2821,20 +2753,16 @@
           <x:t xml:space="preserve">100K/150K rollovers, 250K pops, 500K/750K Super, optional 250K star</x:t>
         </x:is>
       </x:c>
-      <x:c r="K33" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8/10-second circuit windows and a 16/20-second single-attempt Super</x:t>
-        </x:is>
+      <x:c r="K33" s="31" t="str">
+        <x:v>8/10-second circuits; A/B and flashing pops accelerate after 4 seconds. The 16/20-second center-web chase accelerates after 8 seconds.</x:v>
       </x:c>
       <x:c r="L33" s="31" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Center-web Super / expiry / ball end</x:t>
         </x:is>
       </x:c>
-      <x:c r="M33" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Uses underrepresented slings, inlanes, middle rollovers, pops, star, and center web in a readable two-circuit build.</x:t>
-        </x:is>
+      <x:c r="M33" s="31" t="str">
+        <x:v>Purple base GI; available sling/inlane areas pulse and return to GI color when done. Completed pops stay solid. Four-light white web chase and live Super status need machine testing.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -8453,15 +8381,11 @@
           <x:t xml:space="preserve">Spider-Slayer</x:t>
         </x:is>
       </x:c>
-      <x:c r="G24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest polish</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expanding 15-hit hunt: one random category starts lit, every successful lit shot scores and adds another persistent lit category. The fifteenth hit opens the Daily Bugle VUK for a decaying Slayer Jackpot.</x:t>
-        </x:is>
+      <x:c r="G24" s="31" t="str">
+        <x:v>Implemented / reviewed; needs machine test</x:v>
+      </x:c>
+      <x:c r="H24" s="31" t="str">
+        <x:v>Expanding 15-hit hunt with per-category repeat ladders. The fifteenth hit opens a 20-second Daily Bugle VUK countdown (25 with More Time); lit categories continue scoring. Shot Assist scores/counts the first shot twice.</x:v>
       </x:c>
       <x:c r="I24" s="31" t="inlineStr">
         <x:is>
@@ -8499,15 +8423,11 @@
           <x:t xml:space="preserve">Metal-Eating Monster</x:t>
         </x:is>
       </x:c>
-      <x:c r="G25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / needs playtest</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Eight-zone rescue mode. A new safe zone comes under attack every 5 seconds; each attack has an independent 12-second timer. Hits save zones, save reactions bring the next attack in 2 seconds, four saves stop new attacks, and three destroyed zones end the mode.</x:t>
-        </x:is>
+      <x:c r="G25" s="31" t="str">
+        <x:v>Implemented / reviewed; saved-GI fix needs machine test</x:v>
+      </x:c>
+      <x:c r="H25" s="31" t="str">
+        <x:v>Eight-zone rescue: attacks begin every 5s, each has a 12s timer, saves reset the next attack to 2s, four saves stop new attacks, and three destroyed zones end the mode. Attacked zones flash native inserts plus 100% orange GI; saved zones use solid native inserts plus 75% green GI (00BF00); destroyed zones are dark.</x:v>
       </x:c>
       <x:c r="I25" s="31" t="inlineStr">
         <x:is>
@@ -8629,15 +8549,11 @@
           <x:t xml:space="preserve">The Fantastic Fakir</x:t>
         </x:is>
       </x:c>
-      <x:c r="G28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / recent rule update</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2-ball Ruby Heist: one saucer parks a ball and reveals the real Ruby at its mapped upper target; spinners build value and three Ruby Jackpots qualify the Super. A successful Ruby or Super Ruby collect holds the parked saucer ball for 2 seconds before the shared occupancy-checked eject.</x:t>
-        </x:is>
+      <x:c r="G28" s="31" t="str">
+        <x:v>Implemented / reviewed; VUK chase + status fix need machine test</x:v>
+      </x:c>
+      <x:c r="H28" s="31" t="str">
+        <x:v>2-ball Ruby Heist: one saucer parks a ball and opens the gate; the shared VUK route chase guides the live ball until upper entry, where the 10s/15s Ruby timer begins. Spinners build value, three Rubies qualify one Super, and post-Super Rubies continue until multiball ends. Status messages now use the actual Ruby/Super state.</x:v>
       </x:c>
       <x:c r="I28" s="31" t="inlineStr">
         <x:is>
@@ -8676,10 +8592,10 @@
         </x:is>
       </x:c>
       <x:c r="G29" s="31" t="str">
-        <x:v>Implemented / recent Scepter timer display fix</x:v>
+        <x:v>Implemented / reviewed; Scepter wording fix needs machine test</x:v>
       </x:c>
       <x:c r="H29" s="31" t="str">
-        <x:v>Four randomly selected demons appear one at a time every 4s across two webs, two banks, and two pops. Destroying all four starts a 20s scepter phase and opens rooftop access; the VUK scores the 1M Super. The Scepter phase now shows a persistent SCEPTER TIME status (30s with More Time), cancels the prior demon reminder, and displays SHOOT THE VUK or OPTIONAL DEMON - THEN VUK. Lighting uses dim dark-red background GI, independently flashing yellow active demons, and a yellow-only ramp/VUK flash during the scepter phase. Defeat and escape produce the correct summary outcome.</x:v>
+        <x:v>Four randomly selected demons appear one at a time every 4s across two webs, two banks, and two pops. Destroying all four starts a 20s scepter phase and opens rooftop access; the VUK scores the 1M Super. The persistent SCEPTER TIME status uses SUPER AT DAILY BUGLE normally, or KILL THE DEMON, COLLECT THE SUPER while the optional fifth demon remains. Lighting uses dim dark-red background GI, independently flashing yellow active demons, and a yellow-only ramp/VUK flash during the scepter phase. Defeat and escape produce the correct summary outcome.</x:v>
       </x:c>
       <x:c r="I29" s="31" t="inlineStr">
         <x:is>
@@ -8718,10 +8634,10 @@
         </x:is>
       </x:c>
       <x:c r="G30" s="31" t="str">
-        <x:v>Implemented / recent failure-cleanup fix</x:v>
+        <x:v>Implemented / reviewed; flicker/status/gate fix needs machine test</x:v>
       </x:c>
       <x:c r="H30" s="31" t="str">
-        <x:v>Restore six coordinate-based GI regions before the 40-second timer expires. More Jackpots adds a final VUK Blackout Jackpot. Timer failure now enters the centralized failed-summary pipeline, marks Swami played/completed for progression, and clears the villain-running lock after the summary instead of leaving the chapter display at PLAYING.</x:v>
+        <x:v>Restore six coordinate-based GI regions before the 40-second timer expires. Each unrestored 404040 region independently flickers full white for 100ms every random 2–5s; restored regions remain solid white. A persistent CITY TIME status shows seconds and restoration progress, then BLACKOUT AT DAILY BUGLE during the More Jackpots VUK finale. The finale opens the rooftop gate once and uses the shared VUK chase. Timer failure uses the corrected summary/cleanup pipeline.</x:v>
       </x:c>
       <x:c r="I30" s="31" t="inlineStr">
         <x:is>
@@ -8805,15 +8721,11 @@
           <x:t xml:space="preserve">Dr. Noah Boddy</x:t>
         </x:is>
       </x:c>
-      <x:c r="G32" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented / recent rule update</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H32" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Invisible-target search. Upper targets eliminate false lower drops while the upper spinner builds the Secret Jackpot. Each spinner hit also banks the effective 25K increase, or 50K with Bigger Jackpots, in persistent noah_boddy_bonus as INVISIBLE FORTUNE. The hidden target and eliminated false locations persist across rooftop visits. Each entry resets both banks and re-drops prior eliminations; an early exit resets both banks and requires another rooftop entry to continue.</x:t>
-        </x:is>
+      <x:c r="G32" s="31" t="str">
+        <x:v>Implemented / reviewed; lifecycle + VUK chase fix needs machine test</x:v>
+      </x:c>
+      <x:c r="H32" s="31" t="str">
+        <x:v>Invisible-target search. Upper targets eliminate false lower drops while the upper spinner builds the Secret Jackpot. Hidden target and reveal progress persist across rooftop visits. Playing state is 1; both Jackpot success and missed/expired failure finish at completed state 2 with different display messages. The shared VUK chase guides each required rooftop return and stops on entry, result, or cleanup. Rooftop access is requested once from Python.</x:v>
       </x:c>
       <x:c r="I32" s="31" t="inlineStr">
         <x:is>
@@ -8851,15 +8763,11 @@
           <x:t xml:space="preserve">Dr. Magneto</x:t>
         </x:is>
       </x:c>
-      <x:c r="G33" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented redesign / needs playtest</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H33" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cross-feed circuits: left sling/inlane lights right-side A, which lights the left pop; right sling/inlane lights left-side B, which lights the right pop. Hit flashing pops to lock them solid; both solid light the 16-second center-web Super.</x:t>
-        </x:is>
+      <x:c r="G33" s="31" t="str">
+        <x:v>Implemented / reviewed; status + lighting fix needs machine test</x:v>
+      </x:c>
+      <x:c r="H33" s="31" t="str">
+        <x:v>Cross-feed circuits: left sling/inlane lights right-side A and the left pop; right sling/inlane lights left-side B and the right pop. Purple 6030A0 GI underlies pulsing qualifier areas. A/B and flashing pops double pulse speed after 4 seconds. Both completed pops light the center-web Super with a four-step white chase that doubles speed after 8 seconds. Persistent Super status follows the live countdown.</x:v>
       </x:c>
       <x:c r="I33" s="31" t="inlineStr">
         <x:is>
@@ -10534,10 +10442,8 @@
           <x:t xml:space="preserve">The Fantastic Fakir</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Old Ms. Trubble puzzle gameplay repurposed into The Fantastic Fakir's Ruby Heist.</x:t>
-        </x:is>
+      <x:c r="D6" s="31" t="str">
+        <x:v>Old Ms. Trubble puzzle gameplay was replaced by the reviewed Ruby Heist: saucer hold, shared VUK route chase, rooftop Ruby targets, spinner builds, one summed Super, and corrected live status messaging.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10972,10 +10878,8 @@
           <x:t xml:space="preserve">Spider-Slayer</x:t>
         </x:is>
       </x:c>
-      <x:c r="D26" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Originally introduced as a Chapter 5 placeholder; now has the expanding 15-hit hunt and decaying Daily Bugle jackpot implementation.</x:t>
-        </x:is>
+      <x:c r="D26" s="85" t="str">
+        <x:v>Originally a Chapter 5 placeholder; now reviewed as a 15-hit expanding hunt with per-category declining repeat scores and a timed Daily Bugle VUK Jackpot.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -10994,10 +10898,8 @@
           <x:t xml:space="preserve">Metal-Eating Monster</x:t>
         </x:is>
       </x:c>
-      <x:c r="D27" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Originally introduced as a Chapter 5 placeholder; now implemented as an eight-zone overlapping rescue mode with independent destruction timers.</x:t>
-        </x:is>
+      <x:c r="D27" s="85" t="str">
+        <x:v>Originally a Chapter 5 placeholder; now reviewed as an eight-zone overlapping rescue mode. Attacked/saved/destroyed lighting is standardized to 100% flashing orange GI, 75% solid green GI, and dark respectively.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -12061,28 +11963,20 @@
           <x:t xml:space="preserve">Spider-Slayer</x:t>
         </x:is>
       </x:c>
-      <x:c r="E24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">One random shot category starts lit. Each successful lit shot scores 50K and adds another persistent lit category. Hunt Time runs from the first successful hit through the fifteenth, then all build shots shut off and the Daily Bugle VUK lights.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Completes when the Daily Bugle VUK collects the Slayer Jackpot. The winning ball remains held through the villain summary and releases when the summary finishes or is skipped. A drain before collection ends with SLAYER ESCAPED.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H24" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Successful lit shots score 50K; Bigger raises them to 75K. Slayer Jackpot starts at 2M, or 2.5M with Bigger, and decays to a 100K minimum. An unlit VUK visit uses the shared 1.5-second eject.</x:t>
-        </x:is>
+      <x:c r="E24" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F24" s="31" t="str">
+        <x:v>Hit persistent lit categories; each successful hit adds another category. Repeat values decline independently per logical category.</x:v>
+      </x:c>
+      <x:c r="G24" s="31" t="str">
+        <x:v>Slayer Jackpot collected or ball end; an expired VUK countdown closes the gate while lit-category scoring continues.</x:v>
+      </x:c>
+      <x:c r="H24" s="31" t="str">
+        <x:v>15 qualifying hits open the Daily Bugle VUK for 20 seconds (25 with More Time). Shot ladders are 50K/25K/10K/5K, or 75K/50K/25K/10K with Bigger. More Jackpots preserves the full second-hit value; Shot Assist scores/counts the first shot twice.</x:v>
       </x:c>
       <x:c r="I24" s="31" t="str">
-        <x:v>More Jackpots freezes the full jackpot for 10 seconds. More Time halves decay to 50K/sec. Safety Net starts a 10-second save when the VUK lights. Shot Assist makes the first hit add two new categories. The shared Master Vine route chase guides the terminal VUK and clears on collect or teardown; needs machine playtest.</x:v>
+        <x:v>All active categories pulse red; the saucer category uses all six red hole lamps. Summary shows collected Jackpot only and omits Hunt Time until the hunt is completed.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -12124,10 +12018,8 @@
           <x:t xml:space="preserve">Saving a zone scores 250K and resets the next-attack delay to 2 seconds. More Time gives 16-second zone timers; Bigger gives 400K saves; More Jackpots relights each saved zone once for half value; Safety Net is the standard ball save; Shot Assist automatically saves the first zone that reaches 2 seconds.</x:t>
         </x:is>
       </x:c>
-      <x:c r="I25" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented with eight physical zone groups and native-lens attack/save lighting; needs machine playtest.</x:t>
-        </x:is>
+      <x:c r="I25" s="31" t="str">
+        <x:v>Reviewed lighting: attacked zones flash native inserts and 100% orange GI every 250ms; saved zones retain solid native inserts with 75% green GI (00BF00); destroyed zones remain dark.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -12228,25 +12120,17 @@
           <x:t xml:space="preserve">2-ball MB</x:t>
         </x:is>
       </x:c>
-      <x:c r="F28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ruby Heist multiball: a saucer parks one ball and reveals an upper Ruby while the live ball reaches the roof and spinners build the Ruby/Super value. After a successful Ruby or Super collect, the parked ball remains held for 2 seconds before release.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ends when Fakir multiball ends.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ruby Heist: saucers reveal upper rubies; spinners build value; 3 Ruby JPs qualify Super; post-Super rubies continue until multiball ends.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I28" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Improved: persistent Ruby progress, reveal objective, Super-lit status, and a 2-second successful-collect saucer hold using the shared eject service.</x:t>
-        </x:is>
+      <x:c r="F28" s="31" t="str">
+        <x:v>Park a ball in a saucer, follow the VUK chase to the roof, then hit the mapped upper Ruby; spinners build the active award.</x:v>
+      </x:c>
+      <x:c r="G28" s="31" t="str">
+        <x:v>Ends when Fakir multiball returns to one ball.</x:v>
+      </x:c>
+      <x:c r="H28" s="31" t="str">
+        <x:v>Three Ruby Jackpots qualify one Super equal to their combined collected values; post-Super base Rubies continue. The rooftop timer begins only on upper entry.</x:v>
+      </x:c>
+      <x:c r="I28" s="31" t="str">
+        <x:v>Shared green VUK chase runs only while rooftop access is being sought. Live status now reports Ruby/Super state, mapped target, builds, collections, timeouts, and readiness.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -12283,7 +12167,7 @@
         <x:v>Demons appear every 4s and remain active until collected. Jackpots are 200K, 250K, 300K, and 350K. Scepter phase lasts 20s and awards a 1M Super.</x:v>
       </x:c>
       <x:c r="I29" s="31" t="str">
-        <x:v>Dim 401010 background GI; active demons flash yellow every 300ms. The shared Master Vine route chase guides the timed final VUK shot during the scepter phase and clears on collect, timeout, or teardown. More JP adds an independently flashing optional 500K demon. Needs machine playtest.</x:v>
+        <x:v>Dim 401010 background GI; active demons flash yellow every 300ms. The shared Master Vine route chase guides the timed final VUK shot during the scepter phase and clears on collect, timeout, or teardown. Status reads SUPER AT DAILY BUGLE, or KILL THE DEMON, COLLECT THE SUPER while the optional 500K demon remains. Needs machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -12326,7 +12210,7 @@
         </x:is>
       </x:c>
       <x:c r="I30" s="31" t="str">
-        <x:v>Restored regions remain lit. With More Jackpots, the shared Master Vine route chase guides the final 500K Blackout Jackpot at the VUK and clears on collect, timeout, or teardown. Safety Net starts ball save; Shot Assist spots one additional unrestored region. Needs machine regression testing.</x:v>
+        <x:v>Unrestored 404040 regions independently flicker full white for 100ms every random 2–5s; restored regions stay solid white. CITY TIME shows the live countdown and restored count, changing to BLACKOUT AT DAILY BUGLE for the More JP finale. The finale uses one guarded gate-open event and the shared VUK chase. Needs machine regression testing.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -12413,10 +12297,8 @@
           <x:t xml:space="preserve">Upper targets score 25K, or 75K with More Jackpots. Each upper spin increases the displayed Jackpot by 25K, or effectively 50K with Bigger, and banks that increment as persistent INVISIBLE FORTUNE.</x:t>
         </x:is>
       </x:c>
-      <x:c r="I32" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented with persistent cross-visit reveal progress, reconstructed physical drop state, uncapped spinner building, noah_boddy_bonus banking, hurry-up, Case Files, status, and summary values; needs on-machine playtest.</x:t>
-        </x:is>
+      <x:c r="I32" s="31" t="str">
+        <x:v>Persistent cross-visit reveal progress, reconstructed physical drop state, uncapped spinner building, INVISIBLE FORTUNE banking, hurry-up, Case Files, status, and summaries retained. Shared VUK chase runs only while rooftop entry is needed. Success and failure display differently but both mark completed progression. Duplicate YAML gate request removed. Needs machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -12458,10 +12340,8 @@
           <x:t xml:space="preserve">Lit rollover 100K; flashing pop 250K; center-web Super 500K. Bigger Jackpots changes rollover hits to 150K and the Super to 750K.</x:t>
         </x:is>
       </x:c>
-      <x:c r="I33" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">More Jackpots lights the star for 6 seconds and 250K whenever a new objective lights. More Time gives 10-second circuits and a 20-second Super. Safety Net is a 10-second opening save. Shot Assist lights A and B on the first qualifier.</x:t>
-        </x:is>
+      <x:c r="I33" s="31" t="str">
+        <x:v>More Jackpots lights STAR for 6 seconds and 250K whenever a new objective lights. More Time gives 10-second circuits and a 20-second Super. Safety Net is a 10-second opening save. Shot Assist lights A and B on the first qualifier. Purple GI, qualifier-area pulses, 4-second objective acceleration, an 8-second-delayed center-web chase acceleration, and live Super status are implemented; needs machine playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">

</xml_diff>

<commit_message>
more music and zapp fix
</commit_message>
<xml_diff>
--- a/docs/spiderman_1967_50_villain_chapter_plan.xlsx
+++ b/docs/spiderman_1967_50_villain_chapter_plan.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3313b8cce8b04e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Re8ed0d31a08f43b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R6a8c58c188964097"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R1b0956c0b3c144a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R233bc989fbc64ece"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Re2ba4c1aa4ea45ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Raa17dde6de784881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R425ad4d5b97943a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="Rebd86664dc724cc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R11e23c09aa034927"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R07e11370d2784538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R9bfbccb937ac4fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="Ra81896037cee4cf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Reb0c41b0e535425e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="R24ef06a1a8a8465e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="R5ca34f4559584f79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="R44cc960f30e444db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R7c673aebe65d4fef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R5128b519b4164f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="Rc046f837cd0c43a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R16f1c3fcb54b4f9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R39c7ac30dd4f4626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="Raa02d98ccba84d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rb49767a7b0094bea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R77d85c6c0d4c43ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R035f15c4f4544a28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5167,7 +5167,7 @@
     </x:row>
     <x:row r="2" s="26" customFormat="1" ht="30" customHeight="1">
       <x:c r="A2" s="83" t="str">
-        <x:v>Source of truth: current villain_bookends.py and music_control.py/yaml as of 2026-08-23. Bookends own villain/wizard music; music_control owns chapter base music.</x:v>
+        <x:v>Source of truth: ASM67_2026_08_27_1am.zip — current villain_bookends.py and music_control.py/yaml. Bookends own villain/wizard music; music_control owns chapter base music.</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -5176,7 +5176,7 @@
     </x:row>
     <x:row r="3" s="26" customFormat="1" ht="30" customHeight="1">
       <x:c r="A3" s="83" t="str">
-        <x:v>Rule: chapter base themes use longer songs. Villain/wizard songs have at most two uses; maintheme, loop*, and intro_* tracks remain outside villain/wizard gameplay.</x:v>
+        <x:v>Rule: all 67 villain/wizard modes now have unique gameplay songs. maintheme, loop*, and intro_* tracks remain outside villain/wizard gameplay; Song 8 remains within its special-use limit.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -5249,15 +5249,15 @@
           <x:t xml:space="preserve">rat_race</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cyclops; Kingpin / Final Showdown</x:t>
-        </x:is>
+      <x:c r="C8" s="74" t="str">
+        <x:v>Cyclops</x:v>
       </x:c>
       <x:c r="D8" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E8" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="74" t="str">
+        <x:v>Kingpin / Final Showdown reassigned to Song 82.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A9" s="73" t="n">
@@ -5637,15 +5637,15 @@
           <x:t xml:space="preserve">tautwalk</x:t>
         </x:is>
       </x:c>
-      <x:c r="C28" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Electro; Time Showdown</x:t>
-        </x:is>
+      <x:c r="C28" s="74" t="str">
+        <x:v>Electro</x:v>
       </x:c>
       <x:c r="D28" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E28" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E28" s="74" t="str">
+        <x:v>Time-Tossed Showdown reassigned to Song 83.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A29" s="73" t="n">
@@ -5910,15 +5910,15 @@
           <x:t xml:space="preserve">the_hearse</x:t>
         </x:is>
       </x:c>
-      <x:c r="C43" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Doctor Zapp; The Web Tightens</x:t>
-        </x:is>
+      <x:c r="C43" s="74" t="str">
+        <x:v>Doctor Zapp</x:v>
       </x:c>
       <x:c r="D43" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E43" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E43" s="74" t="str">
+        <x:v>The Web Tightens reassigned to Song 84.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A44" s="73" t="n">
@@ -5986,15 +5986,15 @@
           <x:t xml:space="preserve">the_shadows</x:t>
         </x:is>
       </x:c>
-      <x:c r="C47" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The Plutonians; The Molemen</x:t>
-        </x:is>
+      <x:c r="C47" s="74" t="str">
+        <x:v>The Plutonians</x:v>
       </x:c>
       <x:c r="D47" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E47" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E47" s="74" t="str">
+        <x:v>The Molemen reassigned to Song 85.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A48" s="73" t="n">
@@ -6005,15 +6005,15 @@
           <x:t xml:space="preserve">fbi</x:t>
         </x:is>
       </x:c>
-      <x:c r="C48" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Igor; Crime Wave</x:t>
-        </x:is>
+      <x:c r="C48" s="74" t="str">
+        <x:v>Igor</x:v>
       </x:c>
       <x:c r="D48" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E48" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E48" s="74" t="str">
+        <x:v>Crime Wave reassigned to Song 86.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A49" s="73" t="n">
@@ -6081,15 +6081,15 @@
           <x:t xml:space="preserve">motorcycle_circus</x:t>
         </x:is>
       </x:c>
-      <x:c r="C52" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mastermind Trap; Trubble Unleashed</x:t>
-        </x:is>
+      <x:c r="C52" s="74" t="str">
+        <x:v>Mastermind Trap</x:v>
       </x:c>
       <x:c r="D52" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E52" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E52" s="74" t="str">
+        <x:v>Trubble Unleashed reassigned to Song 87.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A53" s="73" t="n">
@@ -6138,15 +6138,15 @@
           <x:t xml:space="preserve">clasical_gas</x:t>
         </x:is>
       </x:c>
-      <x:c r="C55" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fiddler; Sinister Surge</x:t>
-        </x:is>
+      <x:c r="C55" s="74" t="str">
+        <x:v>Fiddler</x:v>
       </x:c>
       <x:c r="D55" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E55" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E55" s="74" t="str">
+        <x:v>Sinister Surge reassigned to Song 88.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A56" s="73" t="n">
@@ -6193,15 +6193,15 @@
           <x:t xml:space="preserve">moon_godess</x:t>
         </x:is>
       </x:c>
-      <x:c r="C58" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pardo; Master Vine</x:t>
-        </x:is>
+      <x:c r="C58" s="74" t="str">
+        <x:v>Pardo</x:v>
       </x:c>
       <x:c r="D58" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E58" s="74" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E58" s="74" t="str">
+        <x:v>Master Vine reassigned to Song 89.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" s="26" customFormat="1" ht="15" customHeight="1">
       <x:c r="A59" s="73" t="n">
@@ -6233,18 +6233,14 @@
           <x:t xml:space="preserve">death_have_no_mercy</x:t>
         </x:is>
       </x:c>
-      <x:c r="C60" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Spider-Slayer; Lost World Invasion</x:t>
-        </x:is>
+      <x:c r="C60" s="74" t="str">
+        <x:v>Spider-Slayer</x:v>
       </x:c>
       <x:c r="D60" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E60" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">New track now integrated.</x:t>
-        </x:is>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E60" s="74" t="str">
+        <x:v>Invasion from Everywhere reassigned to Song 90.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" s="26" customFormat="1" ht="15" customHeight="1">
@@ -6279,18 +6275,14 @@
           <x:t xml:space="preserve">washington_square</x:t>
         </x:is>
       </x:c>
-      <x:c r="C62" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Clive and Blotto; Sir Galahad</x:t>
-        </x:is>
+      <x:c r="C62" s="74" t="str">
+        <x:v>Clive and Blotto</x:v>
       </x:c>
       <x:c r="D62" s="73" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E62" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">New track now integrated.</x:t>
-        </x:is>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E62" s="74" t="str">
+        <x:v>Sir Galahad reassigned to Song 91.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" s="26" customFormat="1" ht="15" customHeight="1">
@@ -6302,18 +6294,14 @@
           <x:t xml:space="preserve">bongo_rock</x:t>
         </x:is>
       </x:c>
-      <x:c r="C63" s="76" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Metal Monster; Bolton and Boomer</x:t>
-        </x:is>
+      <x:c r="C63" s="76" t="str">
+        <x:v>Metal Monster</x:v>
       </x:c>
       <x:c r="D63" s="75" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E63" s="76" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">New track now integrated.</x:t>
-        </x:is>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E63" s="76" t="str">
+        <x:v>Bolton and Boomer reassigned to Song 92.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" s="26" customFormat="1" ht="15" customHeight="1">
@@ -6360,25 +6348,17 @@
           <x:t xml:space="preserve">Sinister Surge</x:t>
         </x:is>
       </x:c>
-      <x:c r="B68" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C68" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">None</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D68" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">50</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E68" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bookend assignment remains active.</x:t>
-        </x:is>
+      <x:c r="B68" s="85" t="str">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="C68" s="85" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D68" s="85" t="str">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="E68" s="85" t="str">
+        <x:v>Bookend assignment updated to Fuzz.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" s="26" customFormat="1" ht="26.399999618530273" customHeight="1">
@@ -6414,25 +6394,17 @@
           <x:t xml:space="preserve">Trubble Unleashed</x:t>
         </x:is>
       </x:c>
-      <x:c r="B70" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">47</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C70" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">None</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D70" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">47</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E70" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bookend assignment remains active.</x:t>
-        </x:is>
+      <x:c r="B70" s="85" t="str">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C70" s="85" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D70" s="85" t="str">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E70" s="85" t="str">
+        <x:v>Bookend assignment updated to Mas Que Nada.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" s="26" customFormat="1" ht="39.599998474121094" customHeight="1">
@@ -6468,25 +6440,17 @@
           <x:t xml:space="preserve">Final Showdown / Kingpin</x:t>
         </x:is>
       </x:c>
-      <x:c r="B72" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C72" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">None</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D72" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E72" s="85" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bookend assignment remains active.</x:t>
-        </x:is>
+      <x:c r="B72" s="85" t="str">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C72" s="85" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D72" s="85" t="str">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E72" s="85" t="str">
+        <x:v>Bookend assignment updated to Rescue Squad.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" s="26" customFormat="1" ht="15" customHeight="1">
@@ -7326,6 +7290,219 @@
       </x:c>
       <x:c r="E123" t="str">
         <x:v>After skill shot and villain summary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>Duplicate-Replacement Assignments</x:v>
+      </x:c>
+      <x:c r="B125"/>
+      <x:c r="C125"/>
+      <x:c r="D125"/>
+      <x:c r="E125"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>Song #</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>Configured Asset</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>Effective Uses</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>rescue_squad</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>Final Showdown / Kingpin</x:v>
+      </x:c>
+      <x:c r="D127" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>Replaces duplicate Song 3; file rescue_squad.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>galatea</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>Time-Tossed Showdown</x:v>
+      </x:c>
+      <x:c r="D128" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>Replaces duplicate Song 23; file galatea.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>uptight</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>The Web Tightens</x:v>
+      </x:c>
+      <x:c r="D129" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>Replaces duplicate Song 38; file uptight.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>monte_carlo</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>The Molemen</x:v>
+      </x:c>
+      <x:c r="D130" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>Replaces duplicate Song 42; file monte_carlo.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>mersey_front</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>Crime Wave</x:v>
+      </x:c>
+      <x:c r="D131" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>Replaces duplicate Song 43; file mersey_front.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>mas_que_nada</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>Trubble Unleashed</x:v>
+      </x:c>
+      <x:c r="D132" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>Replaces duplicate Song 47; file mas_que_nada.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>fuzz</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>Sinister Surge</x:v>
+      </x:c>
+      <x:c r="D133" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>Replaces duplicate Song 50; file fuzz.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>cardova</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>Master Vine</x:v>
+      </x:c>
+      <x:c r="D134" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>Replaces duplicate Song 53; file cardova.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>birds_lament</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>Invasion from Everywhere</x:v>
+      </x:c>
+      <x:c r="D135" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>Replaces duplicate Song 55; file birds_lament.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>come_september</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>Sir Galahad</x:v>
+      </x:c>
+      <x:c r="D136" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>Replaces duplicate Song 57; file come_september.wav.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>runaway</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>Bolton and Boomer</x:v>
+      </x:c>
+      <x:c r="D137" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>Replaces duplicate Song 58; file runaway.wav.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>